<commit_message>
Piano di spesa Tappa Zero: aggiunge il drone per riprese video e diretta live
DJI Mini 4 Pro o Mini 5 Pro, € 400–700: stimato al massimo come il telo del
proiettore. Entra nell'area C, ora «Immagine, media e presentazione»; le voci
successive scalano di un numero. Totale base € 2.882,65.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014EyPNYo6uPPTyzbFJvdbw6
</commit_message>
<xml_diff>
--- a/piano-spesa-tappa-zero-2026/dist/piano-spesa-tappa-zero-2026.xlsx
+++ b/piano-spesa-tappa-zero-2026/dist/piano-spesa-tappa-zero-2026.xlsx
@@ -13,7 +13,7 @@
   </sheets>
   <definedNames>
     <definedName function="false" hidden="false" localSheetId="0" name="_xlnm.Print_Titles" vbProcedure="false">'Piano di spesa'!$10:$10</definedName>
-    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">'Piano di spesa'!$A$10:$P$28</definedName>
+    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">'Piano di spesa'!$A$10:$P$29</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -83,7 +83,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="188" uniqueCount="103">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="198" uniqueCount="106">
   <si>
     <t xml:space="preserve">PIANO DI SPESA · TAPPA ZERO</t>
   </si>
@@ -283,7 +283,7 @@
     <t xml:space="preserve">Voce eventuale: fuori dal totale base.</t>
   </si>
   <si>
-    <t xml:space="preserve">C · Immagine e presentazione</t>
+    <t xml:space="preserve">C · Immagine, media e presentazione</t>
   </si>
   <si>
     <t xml:space="preserve">Wall per foto giocatori</t>
@@ -310,6 +310,15 @@
     <t xml:space="preserve">Prezzo fra € 80 e € 100: messo il massimo per prudenza.</t>
   </si>
   <si>
+    <t xml:space="preserve">Drone per riprese e diretta live</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DJI Mini 4 Pro o Mini 5 Pro per riprese aeree e diretta streaming della tappa.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">€ 400–700 secondo modello e kit: messo il massimo per prudenza.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Tovaglia tavolo presentazione AIFG</t>
   </si>
   <si>
@@ -349,7 +358,7 @@
     <t xml:space="preserve">• Pieghevole A4 (n. 1) e A3 (n. 2) sono alternativi: nel totale base c'è l'A4. Per passare all'A3 invertire «Nel totale» sulle due righe.</t>
   </si>
   <si>
-    <t xml:space="preserve">• Mini vele (n. 8) è voce eventuale, fuori dal totale base. Telo proiettore: € 80–100, messo il massimo per prudenza.</t>
+    <t xml:space="preserve">• Mini vele (n. 8) è voce eventuale, fuori dal totale base. Telo proiettore (€ 80–100) e drone (€ 400–700): messo il massimo per prudenza.</t>
   </si>
   <si>
     <t xml:space="preserve">• Tavoli ristoro: quantità 4 ipotizzata, da confermare. IVA indicata come inclusa solo dove il preventivo lo dice esplicitamente.</t>
@@ -385,7 +394,7 @@
     <t xml:space="preserve">C</t>
   </si>
   <si>
-    <t xml:space="preserve">Immagine e presentazione</t>
+    <t xml:space="preserve">Immagine, media e presentazione</t>
   </si>
   <si>
     <t xml:space="preserve">D</t>
@@ -1542,7 +1551,7 @@
                   <c:v>Allestimento del campo</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>Immagine e presentazione</c:v>
+                  <c:v>Immagine, media e presentazione</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>Punto ristoro</c:v>
@@ -1563,7 +1572,7 @@
                   <c:v>1044</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>679</c:v>
+                  <c:v>1379</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>148</c:v>
@@ -1574,11 +1583,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="77458160"/>
-        <c:axId val="46013591"/>
+        <c:axId val="29939566"/>
+        <c:axId val="93291167"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="77458160"/>
+        <c:axId val="29939566"/>
         <c:scaling>
           <c:orientation val="maxMin"/>
         </c:scaling>
@@ -1610,7 +1619,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="46013591"/>
+        <c:crossAx val="93291167"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1618,7 +1627,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="46013591"/>
+        <c:axId val="93291167"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1650,7 +1659,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="77458160"/>
+        <c:crossAx val="29939566"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1936,7 +1945,7 @@
     <tabColor rgb="FF0072CE"/>
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:P35"/>
+  <dimension ref="A1:P36"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5"/>
@@ -2045,22 +2054,22 @@
     </row>
     <row r="6" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B6" s="7" t="n">
-        <f aca="false">SUMIFS($I$11:$I$28,$L$11:$L$28,"Sì")</f>
-        <v>2182.65</v>
+        <f aca="false">SUMIFS($I$11:$I$29,$L$11:$L$29,"Sì")</f>
+        <v>2882.65</v>
       </c>
       <c r="C6" s="7"/>
       <c r="D6" s="8" t="n">
-        <f aca="false">SUMIFS($I$11:$I$28,$K$11:$K$28,"Opzionale",$L$11:$L$28,"No")</f>
+        <f aca="false">SUMIFS($I$11:$I$29,$K$11:$K$29,"Opzionale",$L$11:$L$29,"No")</f>
         <v>2000</v>
       </c>
       <c r="E6" s="9" t="n">
         <f aca="false">B6+D6</f>
-        <v>4182.65</v>
+        <v>4882.65</v>
       </c>
       <c r="F6" s="9"/>
       <c r="G6" s="9"/>
       <c r="H6" s="10" t="n">
-        <f aca="false">COUNTIFS($K$11:$K$28,"Da definire")</f>
+        <f aca="false">COUNTIFS($K$11:$K$29,"Da definire")</f>
         <v>4</v>
       </c>
       <c r="I6" s="10"/>
@@ -2622,16 +2631,18 @@
       <c r="G21" s="23" t="s">
         <v>30</v>
       </c>
-      <c r="H21" s="24"/>
-      <c r="I21" s="25" t="str">
+      <c r="H21" s="24" t="n">
+        <v>700</v>
+      </c>
+      <c r="I21" s="25" t="n">
         <f aca="false">IF(OR(F21="",H21=""),"",F21*H21)</f>
-        <v/>
+        <v>700</v>
       </c>
       <c r="J21" s="23" t="s">
         <v>44</v>
       </c>
       <c r="K21" s="26" t="s">
-        <v>45</v>
+        <v>72</v>
       </c>
       <c r="L21" s="27" t="s">
         <v>33</v>
@@ -2652,33 +2663,31 @@
         <v>12</v>
       </c>
       <c r="B22" s="33" t="s">
+        <v>66</v>
+      </c>
+      <c r="C22" s="34" t="s">
         <v>78</v>
       </c>
-      <c r="C22" s="34" t="s">
+      <c r="D22" s="35" t="s">
         <v>79</v>
-      </c>
-      <c r="D22" s="35" t="s">
-        <v>80</v>
       </c>
       <c r="E22" s="21"/>
       <c r="F22" s="22" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="G22" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="H22" s="24" t="n">
-        <v>37</v>
-      </c>
-      <c r="I22" s="37" t="n">
+      <c r="H22" s="24"/>
+      <c r="I22" s="37" t="str">
         <f aca="false">IF(OR(F22="",H22=""),"",F22*H22)</f>
-        <v>148</v>
+        <v/>
       </c>
       <c r="J22" s="36" t="s">
         <v>44</v>
       </c>
       <c r="K22" s="38" t="s">
-        <v>72</v>
+        <v>45</v>
       </c>
       <c r="L22" s="39" t="s">
         <v>33</v>
@@ -2691,7 +2700,7 @@
         <v>35</v>
       </c>
       <c r="P22" s="41" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2699,7 +2708,7 @@
         <v>13</v>
       </c>
       <c r="B23" s="18" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="C23" s="19" t="s">
         <v>82</v>
@@ -2714,16 +2723,18 @@
       <c r="G23" s="23" t="s">
         <v>30</v>
       </c>
-      <c r="H23" s="24"/>
-      <c r="I23" s="25" t="str">
+      <c r="H23" s="24" t="n">
+        <v>37</v>
+      </c>
+      <c r="I23" s="25" t="n">
         <f aca="false">IF(OR(F23="",H23=""),"",F23*H23)</f>
-        <v/>
+        <v>148</v>
       </c>
       <c r="J23" s="23" t="s">
         <v>44</v>
       </c>
       <c r="K23" s="26" t="s">
-        <v>45</v>
+        <v>72</v>
       </c>
       <c r="L23" s="27" t="s">
         <v>33</v>
@@ -2743,26 +2754,46 @@
       <c r="A24" s="32" t="n">
         <v>14</v>
       </c>
-      <c r="B24" s="33"/>
-      <c r="C24" s="34"/>
-      <c r="D24" s="35"/>
+      <c r="B24" s="33" t="s">
+        <v>81</v>
+      </c>
+      <c r="C24" s="34" t="s">
+        <v>85</v>
+      </c>
+      <c r="D24" s="35" t="s">
+        <v>86</v>
+      </c>
       <c r="E24" s="21"/>
-      <c r="F24" s="22"/>
-      <c r="G24" s="36"/>
+      <c r="F24" s="22" t="n">
+        <v>4</v>
+      </c>
+      <c r="G24" s="36" t="s">
+        <v>30</v>
+      </c>
       <c r="H24" s="24"/>
       <c r="I24" s="37" t="str">
         <f aca="false">IF(OR(F24="",H24=""),"",F24*H24)</f>
         <v/>
       </c>
-      <c r="J24" s="36"/>
-      <c r="K24" s="38"/>
-      <c r="L24" s="39"/>
-      <c r="M24" s="40"/>
+      <c r="J24" s="36" t="s">
+        <v>44</v>
+      </c>
+      <c r="K24" s="38" t="s">
+        <v>45</v>
+      </c>
+      <c r="L24" s="39" t="s">
+        <v>33</v>
+      </c>
+      <c r="M24" s="40" t="s">
+        <v>34</v>
+      </c>
       <c r="N24" s="29"/>
       <c r="O24" s="30" t="s">
         <v>35</v>
       </c>
-      <c r="P24" s="41"/>
+      <c r="P24" s="41" t="s">
+        <v>87</v>
+      </c>
     </row>
     <row r="25" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="17" t="n">
@@ -2864,56 +2895,81 @@
       </c>
       <c r="P28" s="41"/>
     </row>
-    <row r="29" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="1"/>
-      <c r="B29" s="1"/>
-      <c r="C29" s="42" t="s">
-        <v>85</v>
-      </c>
-      <c r="D29" s="1"/>
-      <c r="E29" s="1"/>
-      <c r="F29" s="1"/>
-      <c r="G29" s="1"/>
-      <c r="H29" s="1"/>
-      <c r="I29" s="43" t="n">
-        <f aca="false">SUMIFS($I$11:$I$28,$L$11:$L$28,"Sì")</f>
-        <v>2182.65</v>
-      </c>
-      <c r="J29" s="1"/>
-      <c r="K29" s="1"/>
-      <c r="L29" s="1"/>
-      <c r="M29" s="1"/>
-      <c r="N29" s="1"/>
-      <c r="O29" s="1"/>
-      <c r="P29" s="1"/>
-    </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B31" s="44" t="s">
-        <v>86</v>
-      </c>
+    <row r="29" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="17" t="n">
+        <v>19</v>
+      </c>
+      <c r="B29" s="18"/>
+      <c r="C29" s="19"/>
+      <c r="D29" s="20"/>
+      <c r="E29" s="21"/>
+      <c r="F29" s="22"/>
+      <c r="G29" s="23"/>
+      <c r="H29" s="24"/>
+      <c r="I29" s="25" t="str">
+        <f aca="false">IF(OR(F29="",H29=""),"",F29*H29)</f>
+        <v/>
+      </c>
+      <c r="J29" s="23"/>
+      <c r="K29" s="26"/>
+      <c r="L29" s="27"/>
+      <c r="M29" s="28"/>
+      <c r="N29" s="29"/>
+      <c r="O29" s="30" t="s">
+        <v>35</v>
+      </c>
+      <c r="P29" s="31"/>
+    </row>
+    <row r="30" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="1"/>
+      <c r="B30" s="1"/>
+      <c r="C30" s="42" t="s">
+        <v>88</v>
+      </c>
+      <c r="D30" s="1"/>
+      <c r="E30" s="1"/>
+      <c r="F30" s="1"/>
+      <c r="G30" s="1"/>
+      <c r="H30" s="1"/>
+      <c r="I30" s="43" t="n">
+        <f aca="false">SUMIFS($I$11:$I$29,$L$11:$L$29,"Sì")</f>
+        <v>2882.65</v>
+      </c>
+      <c r="J30" s="1"/>
+      <c r="K30" s="1"/>
+      <c r="L30" s="1"/>
+      <c r="M30" s="1"/>
+      <c r="N30" s="1"/>
+      <c r="O30" s="1"/>
+      <c r="P30" s="1"/>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B32" s="45" t="s">
-        <v>87</v>
+      <c r="B32" s="44" t="s">
+        <v>89</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B33" s="45" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B34" s="45" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B35" s="45" t="s">
-        <v>90</v>
+        <v>92</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B36" s="45" t="s">
+        <v>93</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A10:P28"/>
+  <autoFilter ref="A10:P29"/>
   <mergeCells count="10">
     <mergeCell ref="B5:C5"/>
     <mergeCell ref="E5:G5"/>
@@ -2926,7 +2982,7 @@
     <mergeCell ref="J6:L6"/>
     <mergeCell ref="M6:N6"/>
   </mergeCells>
-  <conditionalFormatting sqref="K11:K28">
+  <conditionalFormatting sqref="K11:K29">
     <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="19">
       <formula>$K11="Preventivo"</formula>
     </cfRule>
@@ -2943,7 +2999,7 @@
       <formula>$K11="Da definire"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="M11:M28">
+  <conditionalFormatting sqref="M11:M29">
     <cfRule type="expression" priority="7" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="24">
       <formula>$M11="Ordinato"</formula>
     </cfRule>
@@ -2954,21 +3010,21 @@
       <formula>$M11="Pagato"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I11:I28">
+  <conditionalFormatting sqref="I11:I29">
     <cfRule type="expression" priority="10" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="27">
       <formula>$L11="No"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="3">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="K11:K28" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="K11:K29" type="list">
       <formula1>"Preventivo,Stima,Opzionale,Alternativa,Da definire"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="L11:L28" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="L11:L29" type="list">
       <formula1>"Sì,No"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="M11:M28" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="M11:M29" type="list">
       <formula1>"Da ordinare,Ordinato,Consegnato,Pagato"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -3008,7 +3064,7 @@
     <row r="1" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1"/>
       <c r="B1" s="46" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
@@ -3019,7 +3075,7 @@
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1"/>
       <c r="B2" s="47" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
@@ -3033,7 +3089,7 @@
         <v>12</v>
       </c>
       <c r="C4" s="48" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="D4" s="48" t="s">
         <v>3</v>
@@ -3045,26 +3101,26 @@
         <v>19</v>
       </c>
       <c r="G4" s="48" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="50" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="B5" s="51" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="C5" s="52" t="n">
-        <f aca="false">COUNTIFS('Piano di spesa'!$B$11:$B$28,"A · Stampa e comunicazione")</f>
+        <f aca="false">COUNTIFS('Piano di spesa'!$B$11:$B$29,"A · Stampa e comunicazione")</f>
         <v>4</v>
       </c>
       <c r="D5" s="53" t="n">
-        <f aca="false">SUMIFS('Piano di spesa'!$I$11:$I$28,'Piano di spesa'!$B$11:$B$28,"A · Stampa e comunicazione",'Piano di spesa'!$L$11:$L$28,"Sì")</f>
+        <f aca="false">SUMIFS('Piano di spesa'!$I$11:$I$29,'Piano di spesa'!$B$11:$B$29,"A · Stampa e comunicazione",'Piano di spesa'!$L$11:$L$29,"Sì")</f>
         <v>311.65</v>
       </c>
       <c r="E5" s="54" t="n">
-        <f aca="false">SUMIFS('Piano di spesa'!$I$11:$I$28,'Piano di spesa'!$B$11:$B$28,"A · Stampa e comunicazione",'Piano di spesa'!$K$11:$K$28,"Opzionale",'Piano di spesa'!$L$11:$L$28,"No")</f>
+        <f aca="false">SUMIFS('Piano di spesa'!$I$11:$I$29,'Piano di spesa'!$B$11:$B$29,"A · Stampa e comunicazione",'Piano di spesa'!$K$11:$K$29,"Opzionale",'Piano di spesa'!$L$11:$L$29,"No")</f>
         <v>0</v>
       </c>
       <c r="F5" s="54" t="n">
@@ -3073,26 +3129,26 @@
       </c>
       <c r="G5" s="55" t="n">
         <f aca="false">IF($D$9=0,0,D5/$D$9)</f>
-        <v>0.142785146496232</v>
+        <v>0.108112327198932</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="50" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="B6" s="51" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="C6" s="52" t="n">
-        <f aca="false">COUNTIFS('Piano di spesa'!$B$11:$B$28,"B · Allestimento del campo")</f>
+        <f aca="false">COUNTIFS('Piano di spesa'!$B$11:$B$29,"B · Allestimento del campo")</f>
         <v>4</v>
       </c>
       <c r="D6" s="53" t="n">
-        <f aca="false">SUMIFS('Piano di spesa'!$I$11:$I$28,'Piano di spesa'!$B$11:$B$28,"B · Allestimento del campo",'Piano di spesa'!$L$11:$L$28,"Sì")</f>
+        <f aca="false">SUMIFS('Piano di spesa'!$I$11:$I$29,'Piano di spesa'!$B$11:$B$29,"B · Allestimento del campo",'Piano di spesa'!$L$11:$L$29,"Sì")</f>
         <v>1044</v>
       </c>
       <c r="E6" s="54" t="n">
-        <f aca="false">SUMIFS('Piano di spesa'!$I$11:$I$28,'Piano di spesa'!$B$11:$B$28,"B · Allestimento del campo",'Piano di spesa'!$K$11:$K$28,"Opzionale",'Piano di spesa'!$L$11:$L$28,"No")</f>
+        <f aca="false">SUMIFS('Piano di spesa'!$I$11:$I$29,'Piano di spesa'!$B$11:$B$29,"B · Allestimento del campo",'Piano di spesa'!$K$11:$K$29,"Opzionale",'Piano di spesa'!$L$11:$L$29,"No")</f>
         <v>2000</v>
       </c>
       <c r="F6" s="54" t="n">
@@ -3101,54 +3157,54 @@
       </c>
       <c r="G6" s="55" t="n">
         <f aca="false">IF($D$9=0,0,D6/$D$9)</f>
-        <v>0.478317641399217</v>
+        <v>0.362166756283281</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="50" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="B7" s="51" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="C7" s="52" t="n">
-        <f aca="false">COUNTIFS('Piano di spesa'!$B$11:$B$28,"C · Immagine e presentazione")</f>
-        <v>3</v>
+        <f aca="false">COUNTIFS('Piano di spesa'!$B$11:$B$29,"C · Immagine, media e presentazione")</f>
+        <v>4</v>
       </c>
       <c r="D7" s="53" t="n">
-        <f aca="false">SUMIFS('Piano di spesa'!$I$11:$I$28,'Piano di spesa'!$B$11:$B$28,"C · Immagine e presentazione",'Piano di spesa'!$L$11:$L$28,"Sì")</f>
-        <v>679</v>
+        <f aca="false">SUMIFS('Piano di spesa'!$I$11:$I$29,'Piano di spesa'!$B$11:$B$29,"C · Immagine, media e presentazione",'Piano di spesa'!$L$11:$L$29,"Sì")</f>
+        <v>1379</v>
       </c>
       <c r="E7" s="54" t="n">
-        <f aca="false">SUMIFS('Piano di spesa'!$I$11:$I$28,'Piano di spesa'!$B$11:$B$28,"C · Immagine e presentazione",'Piano di spesa'!$K$11:$K$28,"Opzionale",'Piano di spesa'!$L$11:$L$28,"No")</f>
+        <f aca="false">SUMIFS('Piano di spesa'!$I$11:$I$29,'Piano di spesa'!$B$11:$B$29,"C · Immagine, media e presentazione",'Piano di spesa'!$K$11:$K$29,"Opzionale",'Piano di spesa'!$L$11:$L$29,"No")</f>
         <v>0</v>
       </c>
       <c r="F7" s="54" t="n">
         <f aca="false">D7+E7</f>
-        <v>679</v>
+        <v>1379</v>
       </c>
       <c r="G7" s="55" t="n">
         <f aca="false">IF($D$9=0,0,D7/$D$9)</f>
-        <v>0.311089730373628</v>
+        <v>0.47837926907533</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="50" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="B8" s="51" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="C8" s="52" t="n">
-        <f aca="false">COUNTIFS('Piano di spesa'!$B$11:$B$28,"D · Punto ristoro")</f>
+        <f aca="false">COUNTIFS('Piano di spesa'!$B$11:$B$29,"D · Punto ristoro")</f>
         <v>2</v>
       </c>
       <c r="D8" s="53" t="n">
-        <f aca="false">SUMIFS('Piano di spesa'!$I$11:$I$28,'Piano di spesa'!$B$11:$B$28,"D · Punto ristoro",'Piano di spesa'!$L$11:$L$28,"Sì")</f>
+        <f aca="false">SUMIFS('Piano di spesa'!$I$11:$I$29,'Piano di spesa'!$B$11:$B$29,"D · Punto ristoro",'Piano di spesa'!$L$11:$L$29,"Sì")</f>
         <v>148</v>
       </c>
       <c r="E8" s="54" t="n">
-        <f aca="false">SUMIFS('Piano di spesa'!$I$11:$I$28,'Piano di spesa'!$B$11:$B$28,"D · Punto ristoro",'Piano di spesa'!$K$11:$K$28,"Opzionale",'Piano di spesa'!$L$11:$L$28,"No")</f>
+        <f aca="false">SUMIFS('Piano di spesa'!$I$11:$I$29,'Piano di spesa'!$B$11:$B$29,"D · Punto ristoro",'Piano di spesa'!$K$11:$K$29,"Opzionale",'Piano di spesa'!$L$11:$L$29,"No")</f>
         <v>0</v>
       </c>
       <c r="F8" s="54" t="n">
@@ -3157,7 +3213,7 @@
       </c>
       <c r="G8" s="55" t="n">
         <f aca="false">IF($D$9=0,0,D8/$D$9)</f>
-        <v>0.0678074817309234</v>
+        <v>0.0513416474424575</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3167,11 +3223,11 @@
       </c>
       <c r="C9" s="57" t="n">
         <f aca="false">SUM(C5:C8)</f>
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D9" s="58" t="n">
         <f aca="false">SUM(D5:D8)</f>
-        <v>2182.65</v>
+        <v>2882.65</v>
       </c>
       <c r="E9" s="59" t="n">
         <f aca="false">SUM(E5:E8)</f>
@@ -3179,7 +3235,7 @@
       </c>
       <c r="F9" s="59" t="n">
         <f aca="false">SUM(F5:F8)</f>
-        <v>4182.65</v>
+        <v>4882.65</v>
       </c>
       <c r="G9" s="60" t="n">
         <f aca="false">IF($D$9=0,0,SUM(G5:G8))</f>

</xml_diff>

<commit_message>
Piano di spesa Tappa Zero: ragazze immagine, via prossimi passi e riquadri di sintesi
- Aggiunge le ragazze immagine (€ 300) nell'area D, ora «Accoglienza e punto
  ristoro». Totale base € 3.182,65.
- Toglie il blocco «Prossimi passi» dall'ultima pagina di dettaglio e i tre
  riquadri in fondo alla pagina 2; la sintesi resta centrata sulla pagina.
- Riepilogo: area e fornitore sulla stessa riga del nome, così le 15 voci
  stanno in una pagina.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014EyPNYo6uPPTyzbFJvdbw6
</commit_message>
<xml_diff>
--- a/piano-spesa-tappa-zero-2026/dist/piano-spesa-tappa-zero-2026.xlsx
+++ b/piano-spesa-tappa-zero-2026/dist/piano-spesa-tappa-zero-2026.xlsx
@@ -13,7 +13,7 @@
   </sheets>
   <definedNames>
     <definedName function="false" hidden="false" localSheetId="0" name="_xlnm.Print_Titles" vbProcedure="false">'Piano di spesa'!$10:$10</definedName>
-    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">'Piano di spesa'!$A$10:$P$29</definedName>
+    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">'Piano di spesa'!$A$10:$P$30</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -83,7 +83,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="198" uniqueCount="106">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="207" uniqueCount="109">
   <si>
     <t xml:space="preserve">PIANO DI SPESA · TAPPA ZERO</t>
   </si>
@@ -328,7 +328,7 @@
     <t xml:space="preserve">Prezzo da richiedere.</t>
   </si>
   <si>
-    <t xml:space="preserve">D · Punto ristoro</t>
+    <t xml:space="preserve">D · Accoglienza e punto ristoro</t>
   </si>
   <si>
     <t xml:space="preserve">Tavoli pieghevoli</t>
@@ -349,6 +349,15 @@
     <t xml:space="preserve">Costo da verificare.</t>
   </si>
   <si>
+    <t xml:space="preserve">Ragazze immagine</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Servizio di ragazze immagine per l'accoglienza e le premiazioni del weekend.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">servizio</t>
+  </si>
+  <si>
     <t xml:space="preserve">TOTALE BASE (voci «Nel totale» = Sì)</t>
   </si>
   <si>
@@ -400,7 +409,7 @@
     <t xml:space="preserve">D</t>
   </si>
   <si>
-    <t xml:space="preserve">Punto ristoro</t>
+    <t xml:space="preserve">Accoglienza e punto ristoro</t>
   </si>
 </sst>
 </file>
@@ -1554,7 +1563,7 @@
                   <c:v>Immagine, media e presentazione</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>Punto ristoro</c:v>
+                  <c:v>Accoglienza e punto ristoro</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -1575,7 +1584,7 @@
                   <c:v>1379</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>148</c:v>
+                  <c:v>448</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1583,11 +1592,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="29939566"/>
-        <c:axId val="93291167"/>
+        <c:axId val="94149724"/>
+        <c:axId val="81542354"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="29939566"/>
+        <c:axId val="94149724"/>
         <c:scaling>
           <c:orientation val="maxMin"/>
         </c:scaling>
@@ -1619,7 +1628,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="93291167"/>
+        <c:crossAx val="81542354"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1627,7 +1636,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="93291167"/>
+        <c:axId val="81542354"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1659,7 +1668,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="29939566"/>
+        <c:crossAx val="94149724"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1945,7 +1954,7 @@
     <tabColor rgb="FF0072CE"/>
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:P36"/>
+  <dimension ref="A1:P37"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5"/>
@@ -2054,22 +2063,22 @@
     </row>
     <row r="6" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B6" s="7" t="n">
-        <f aca="false">SUMIFS($I$11:$I$29,$L$11:$L$29,"Sì")</f>
-        <v>2882.65</v>
+        <f aca="false">SUMIFS($I$11:$I$30,$L$11:$L$30,"Sì")</f>
+        <v>3182.65</v>
       </c>
       <c r="C6" s="7"/>
       <c r="D6" s="8" t="n">
-        <f aca="false">SUMIFS($I$11:$I$29,$K$11:$K$29,"Opzionale",$L$11:$L$29,"No")</f>
+        <f aca="false">SUMIFS($I$11:$I$30,$K$11:$K$30,"Opzionale",$L$11:$L$30,"No")</f>
         <v>2000</v>
       </c>
       <c r="E6" s="9" t="n">
         <f aca="false">B6+D6</f>
-        <v>4882.65</v>
+        <v>5182.65</v>
       </c>
       <c r="F6" s="9"/>
       <c r="G6" s="9"/>
       <c r="H6" s="10" t="n">
-        <f aca="false">COUNTIFS($K$11:$K$29,"Da definire")</f>
+        <f aca="false">COUNTIFS($K$11:$K$30,"Da definire")</f>
         <v>4</v>
       </c>
       <c r="I6" s="10"/>
@@ -2799,21 +2808,41 @@
       <c r="A25" s="17" t="n">
         <v>15</v>
       </c>
-      <c r="B25" s="18"/>
-      <c r="C25" s="19"/>
-      <c r="D25" s="20"/>
+      <c r="B25" s="18" t="s">
+        <v>81</v>
+      </c>
+      <c r="C25" s="19" t="s">
+        <v>88</v>
+      </c>
+      <c r="D25" s="20" t="s">
+        <v>89</v>
+      </c>
       <c r="E25" s="21"/>
-      <c r="F25" s="22"/>
-      <c r="G25" s="23"/>
-      <c r="H25" s="24"/>
-      <c r="I25" s="25" t="str">
+      <c r="F25" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="G25" s="23" t="s">
+        <v>90</v>
+      </c>
+      <c r="H25" s="24" t="n">
+        <v>300</v>
+      </c>
+      <c r="I25" s="25" t="n">
         <f aca="false">IF(OR(F25="",H25=""),"",F25*H25)</f>
-        <v/>
-      </c>
-      <c r="J25" s="23"/>
-      <c r="K25" s="26"/>
-      <c r="L25" s="27"/>
-      <c r="M25" s="28"/>
+        <v>300</v>
+      </c>
+      <c r="J25" s="23" t="s">
+        <v>44</v>
+      </c>
+      <c r="K25" s="26" t="s">
+        <v>32</v>
+      </c>
+      <c r="L25" s="27" t="s">
+        <v>33</v>
+      </c>
+      <c r="M25" s="28" t="s">
+        <v>34</v>
+      </c>
       <c r="N25" s="29"/>
       <c r="O25" s="30" t="s">
         <v>35</v>
@@ -2920,56 +2949,81 @@
       </c>
       <c r="P29" s="31"/>
     </row>
-    <row r="30" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="1"/>
-      <c r="B30" s="1"/>
-      <c r="C30" s="42" t="s">
-        <v>88</v>
-      </c>
-      <c r="D30" s="1"/>
-      <c r="E30" s="1"/>
-      <c r="F30" s="1"/>
-      <c r="G30" s="1"/>
-      <c r="H30" s="1"/>
-      <c r="I30" s="43" t="n">
-        <f aca="false">SUMIFS($I$11:$I$29,$L$11:$L$29,"Sì")</f>
-        <v>2882.65</v>
-      </c>
-      <c r="J30" s="1"/>
-      <c r="K30" s="1"/>
-      <c r="L30" s="1"/>
-      <c r="M30" s="1"/>
-      <c r="N30" s="1"/>
-      <c r="O30" s="1"/>
-      <c r="P30" s="1"/>
-    </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B32" s="44" t="s">
-        <v>89</v>
-      </c>
+    <row r="30" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="32" t="n">
+        <v>20</v>
+      </c>
+      <c r="B30" s="33"/>
+      <c r="C30" s="34"/>
+      <c r="D30" s="35"/>
+      <c r="E30" s="21"/>
+      <c r="F30" s="22"/>
+      <c r="G30" s="36"/>
+      <c r="H30" s="24"/>
+      <c r="I30" s="37" t="str">
+        <f aca="false">IF(OR(F30="",H30=""),"",F30*H30)</f>
+        <v/>
+      </c>
+      <c r="J30" s="36"/>
+      <c r="K30" s="38"/>
+      <c r="L30" s="39"/>
+      <c r="M30" s="40"/>
+      <c r="N30" s="29"/>
+      <c r="O30" s="30" t="s">
+        <v>35</v>
+      </c>
+      <c r="P30" s="41"/>
+    </row>
+    <row r="31" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="1"/>
+      <c r="B31" s="1"/>
+      <c r="C31" s="42" t="s">
+        <v>91</v>
+      </c>
+      <c r="D31" s="1"/>
+      <c r="E31" s="1"/>
+      <c r="F31" s="1"/>
+      <c r="G31" s="1"/>
+      <c r="H31" s="1"/>
+      <c r="I31" s="43" t="n">
+        <f aca="false">SUMIFS($I$11:$I$30,$L$11:$L$30,"Sì")</f>
+        <v>3182.65</v>
+      </c>
+      <c r="J31" s="1"/>
+      <c r="K31" s="1"/>
+      <c r="L31" s="1"/>
+      <c r="M31" s="1"/>
+      <c r="N31" s="1"/>
+      <c r="O31" s="1"/>
+      <c r="P31" s="1"/>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B33" s="45" t="s">
-        <v>90</v>
+      <c r="B33" s="44" t="s">
+        <v>92</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B34" s="45" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B35" s="45" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B36" s="45" t="s">
-        <v>93</v>
+        <v>95</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B37" s="45" t="s">
+        <v>96</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A10:P29"/>
+  <autoFilter ref="A10:P30"/>
   <mergeCells count="10">
     <mergeCell ref="B5:C5"/>
     <mergeCell ref="E5:G5"/>
@@ -2982,7 +3036,7 @@
     <mergeCell ref="J6:L6"/>
     <mergeCell ref="M6:N6"/>
   </mergeCells>
-  <conditionalFormatting sqref="K11:K29">
+  <conditionalFormatting sqref="K11:K30">
     <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="19">
       <formula>$K11="Preventivo"</formula>
     </cfRule>
@@ -2999,7 +3053,7 @@
       <formula>$K11="Da definire"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="M11:M29">
+  <conditionalFormatting sqref="M11:M30">
     <cfRule type="expression" priority="7" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="24">
       <formula>$M11="Ordinato"</formula>
     </cfRule>
@@ -3010,21 +3064,21 @@
       <formula>$M11="Pagato"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I11:I29">
+  <conditionalFormatting sqref="I11:I30">
     <cfRule type="expression" priority="10" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="27">
       <formula>$L11="No"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="3">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="K11:K29" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="K11:K30" type="list">
       <formula1>"Preventivo,Stima,Opzionale,Alternativa,Da definire"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="L11:L29" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="L11:L30" type="list">
       <formula1>"Sì,No"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="M11:M29" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="M11:M30" type="list">
       <formula1>"Da ordinare,Ordinato,Consegnato,Pagato"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -3064,7 +3118,7 @@
     <row r="1" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1"/>
       <c r="B1" s="46" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
@@ -3075,7 +3129,7 @@
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1"/>
       <c r="B2" s="47" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
@@ -3089,7 +3143,7 @@
         <v>12</v>
       </c>
       <c r="C4" s="48" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="D4" s="48" t="s">
         <v>3</v>
@@ -3101,26 +3155,26 @@
         <v>19</v>
       </c>
       <c r="G4" s="48" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="50" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="B5" s="51" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="C5" s="52" t="n">
-        <f aca="false">COUNTIFS('Piano di spesa'!$B$11:$B$29,"A · Stampa e comunicazione")</f>
+        <f aca="false">COUNTIFS('Piano di spesa'!$B$11:$B$30,"A · Stampa e comunicazione")</f>
         <v>4</v>
       </c>
       <c r="D5" s="53" t="n">
-        <f aca="false">SUMIFS('Piano di spesa'!$I$11:$I$29,'Piano di spesa'!$B$11:$B$29,"A · Stampa e comunicazione",'Piano di spesa'!$L$11:$L$29,"Sì")</f>
+        <f aca="false">SUMIFS('Piano di spesa'!$I$11:$I$30,'Piano di spesa'!$B$11:$B$30,"A · Stampa e comunicazione",'Piano di spesa'!$L$11:$L$30,"Sì")</f>
         <v>311.65</v>
       </c>
       <c r="E5" s="54" t="n">
-        <f aca="false">SUMIFS('Piano di spesa'!$I$11:$I$29,'Piano di spesa'!$B$11:$B$29,"A · Stampa e comunicazione",'Piano di spesa'!$K$11:$K$29,"Opzionale",'Piano di spesa'!$L$11:$L$29,"No")</f>
+        <f aca="false">SUMIFS('Piano di spesa'!$I$11:$I$30,'Piano di spesa'!$B$11:$B$30,"A · Stampa e comunicazione",'Piano di spesa'!$K$11:$K$30,"Opzionale",'Piano di spesa'!$L$11:$L$30,"No")</f>
         <v>0</v>
       </c>
       <c r="F5" s="54" t="n">
@@ -3129,26 +3183,26 @@
       </c>
       <c r="G5" s="55" t="n">
         <f aca="false">IF($D$9=0,0,D5/$D$9)</f>
-        <v>0.108112327198932</v>
+        <v>0.0979215433679481</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="50" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="B6" s="51" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="C6" s="52" t="n">
-        <f aca="false">COUNTIFS('Piano di spesa'!$B$11:$B$29,"B · Allestimento del campo")</f>
+        <f aca="false">COUNTIFS('Piano di spesa'!$B$11:$B$30,"B · Allestimento del campo")</f>
         <v>4</v>
       </c>
       <c r="D6" s="53" t="n">
-        <f aca="false">SUMIFS('Piano di spesa'!$I$11:$I$29,'Piano di spesa'!$B$11:$B$29,"B · Allestimento del campo",'Piano di spesa'!$L$11:$L$29,"Sì")</f>
+        <f aca="false">SUMIFS('Piano di spesa'!$I$11:$I$30,'Piano di spesa'!$B$11:$B$30,"B · Allestimento del campo",'Piano di spesa'!$L$11:$L$30,"Sì")</f>
         <v>1044</v>
       </c>
       <c r="E6" s="54" t="n">
-        <f aca="false">SUMIFS('Piano di spesa'!$I$11:$I$29,'Piano di spesa'!$B$11:$B$29,"B · Allestimento del campo",'Piano di spesa'!$K$11:$K$29,"Opzionale",'Piano di spesa'!$L$11:$L$29,"No")</f>
+        <f aca="false">SUMIFS('Piano di spesa'!$I$11:$I$30,'Piano di spesa'!$B$11:$B$30,"B · Allestimento del campo",'Piano di spesa'!$K$11:$K$30,"Opzionale",'Piano di spesa'!$L$11:$L$30,"No")</f>
         <v>2000</v>
       </c>
       <c r="F6" s="54" t="n">
@@ -3157,26 +3211,26 @@
       </c>
       <c r="G6" s="55" t="n">
         <f aca="false">IF($D$9=0,0,D6/$D$9)</f>
-        <v>0.362166756283281</v>
+        <v>0.328028529684383</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="50" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="B7" s="51" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="C7" s="52" t="n">
-        <f aca="false">COUNTIFS('Piano di spesa'!$B$11:$B$29,"C · Immagine, media e presentazione")</f>
+        <f aca="false">COUNTIFS('Piano di spesa'!$B$11:$B$30,"C · Immagine, media e presentazione")</f>
         <v>4</v>
       </c>
       <c r="D7" s="53" t="n">
-        <f aca="false">SUMIFS('Piano di spesa'!$I$11:$I$29,'Piano di spesa'!$B$11:$B$29,"C · Immagine, media e presentazione",'Piano di spesa'!$L$11:$L$29,"Sì")</f>
+        <f aca="false">SUMIFS('Piano di spesa'!$I$11:$I$30,'Piano di spesa'!$B$11:$B$30,"C · Immagine, media e presentazione",'Piano di spesa'!$L$11:$L$30,"Sì")</f>
         <v>1379</v>
       </c>
       <c r="E7" s="54" t="n">
-        <f aca="false">SUMIFS('Piano di spesa'!$I$11:$I$29,'Piano di spesa'!$B$11:$B$29,"C · Immagine, media e presentazione",'Piano di spesa'!$K$11:$K$29,"Opzionale",'Piano di spesa'!$L$11:$L$29,"No")</f>
+        <f aca="false">SUMIFS('Piano di spesa'!$I$11:$I$30,'Piano di spesa'!$B$11:$B$30,"C · Immagine, media e presentazione",'Piano di spesa'!$K$11:$K$30,"Opzionale",'Piano di spesa'!$L$11:$L$30,"No")</f>
         <v>0</v>
       </c>
       <c r="F7" s="54" t="n">
@@ -3185,35 +3239,35 @@
       </c>
       <c r="G7" s="55" t="n">
         <f aca="false">IF($D$9=0,0,D7/$D$9)</f>
-        <v>0.47837926907533</v>
+        <v>0.43328672647008</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="50" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="B8" s="51" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="C8" s="52" t="n">
-        <f aca="false">COUNTIFS('Piano di spesa'!$B$11:$B$29,"D · Punto ristoro")</f>
-        <v>2</v>
+        <f aca="false">COUNTIFS('Piano di spesa'!$B$11:$B$30,"D · Accoglienza e punto ristoro")</f>
+        <v>3</v>
       </c>
       <c r="D8" s="53" t="n">
-        <f aca="false">SUMIFS('Piano di spesa'!$I$11:$I$29,'Piano di spesa'!$B$11:$B$29,"D · Punto ristoro",'Piano di spesa'!$L$11:$L$29,"Sì")</f>
-        <v>148</v>
+        <f aca="false">SUMIFS('Piano di spesa'!$I$11:$I$30,'Piano di spesa'!$B$11:$B$30,"D · Accoglienza e punto ristoro",'Piano di spesa'!$L$11:$L$30,"Sì")</f>
+        <v>448</v>
       </c>
       <c r="E8" s="54" t="n">
-        <f aca="false">SUMIFS('Piano di spesa'!$I$11:$I$29,'Piano di spesa'!$B$11:$B$29,"D · Punto ristoro",'Piano di spesa'!$K$11:$K$29,"Opzionale",'Piano di spesa'!$L$11:$L$29,"No")</f>
+        <f aca="false">SUMIFS('Piano di spesa'!$I$11:$I$30,'Piano di spesa'!$B$11:$B$30,"D · Accoglienza e punto ristoro",'Piano di spesa'!$K$11:$K$30,"Opzionale",'Piano di spesa'!$L$11:$L$30,"No")</f>
         <v>0</v>
       </c>
       <c r="F8" s="54" t="n">
         <f aca="false">D8+E8</f>
-        <v>148</v>
+        <v>448</v>
       </c>
       <c r="G8" s="55" t="n">
         <f aca="false">IF($D$9=0,0,D8/$D$9)</f>
-        <v>0.0513416474424575</v>
+        <v>0.140763200477589</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3223,11 +3277,11 @@
       </c>
       <c r="C9" s="57" t="n">
         <f aca="false">SUM(C5:C8)</f>
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D9" s="58" t="n">
         <f aca="false">SUM(D5:D8)</f>
-        <v>2882.65</v>
+        <v>3182.65</v>
       </c>
       <c r="E9" s="59" t="n">
         <f aca="false">SUM(E5:E8)</f>
@@ -3235,7 +3289,7 @@
       </c>
       <c r="F9" s="59" t="n">
         <f aca="false">SUM(F5:F8)</f>
-        <v>4882.65</v>
+        <v>5182.65</v>
       </c>
       <c r="G9" s="60" t="n">
         <f aca="false">IF($D$9=0,0,SUM(G5:G8))</f>

</xml_diff>

<commit_message>
Piano di spesa Tappa Zero: area Organizzazione e staff e altre voci
- Nuova area E «Organizzazione e staff»: radioline (10), abbigliamento staff
  (polo, maglia, pantalone), cassa con microfono per le partenze (€ 70),
  timer per partenza (€ 80).
- Sedie per gazebo (€ 70) nell'area D, roll up segreteria come opzionale
  nell'area C. Voci rinumerate per area. Totale base € 3.402,65.
- Pagine di dettaglio e numerazione ricavate dalle aree; riepilogo per area
  dell'Excel dimensionato sul numero di aree. Scheda voce più compatta:
  l'IVA compare sotto il totale solo quando è nota.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014EyPNYo6uPPTyzbFJvdbw6
</commit_message>
<xml_diff>
--- a/piano-spesa-tappa-zero-2026/dist/piano-spesa-tappa-zero-2026.xlsx
+++ b/piano-spesa-tappa-zero-2026/dist/piano-spesa-tappa-zero-2026.xlsx
@@ -13,7 +13,7 @@
   </sheets>
   <definedNames>
     <definedName function="false" hidden="false" localSheetId="0" name="_xlnm.Print_Titles" vbProcedure="false">'Piano di spesa'!$10:$10</definedName>
-    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">'Piano di spesa'!$A$10:$P$30</definedName>
+    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">'Piano di spesa'!$A$10:$P$36</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -83,7 +83,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="207" uniqueCount="109">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="267" uniqueCount="129">
   <si>
     <t xml:space="preserve">PIANO DI SPESA · TAPPA ZERO</t>
   </si>
@@ -310,7 +310,7 @@
     <t xml:space="preserve">Prezzo fra € 80 e € 100: messo il massimo per prudenza.</t>
   </si>
   <si>
-    <t xml:space="preserve">Drone per riprese e diretta live</t>
+    <t xml:space="preserve">Drone riprese e diretta</t>
   </si>
   <si>
     <t xml:space="preserve">DJI Mini 4 Pro o Mini 5 Pro per riprese aeree e diretta streaming della tappa.</t>
@@ -319,15 +319,24 @@
     <t xml:space="preserve">€ 400–700 secondo modello e kit: messo il massimo per prudenza.</t>
   </si>
   <si>
-    <t xml:space="preserve">Tovaglia tavolo presentazione AIFG</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tovaglia personalizzata per il tavolo della presentazione AIFG.</t>
+    <t xml:space="preserve">Tovaglia tavolo AIFG</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tovaglia personalizzata per il tavolo della presentazione.</t>
   </si>
   <si>
     <t xml:space="preserve">Prezzo da richiedere.</t>
   </si>
   <si>
+    <t xml:space="preserve">Roll up segreteria</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Roll up per l'area segreteria e iscrizioni.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Voce eventuale: quantità e prezzo da definire.</t>
+  </si>
+  <si>
     <t xml:space="preserve">D · Accoglienza e punto ristoro</t>
   </si>
   <si>
@@ -358,6 +367,51 @@
     <t xml:space="preserve">servizio</t>
   </si>
   <si>
+    <t xml:space="preserve">Sedie per gazebo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sedie per i gazebo dell'accoglienza e della segreteria.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Verificare quante sedie comprende la fornitura.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">E · Organizzazione e staff</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Radioline ricetrasmittenti</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Radio per il collegamento fra segreteria, starter e staff sul percorso.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Prezzo da definire.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Abbigliamento staff</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Polo, maglia e pantalone per lo staff della tappa.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">kit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Quantità per capo e prezzo da definire in base allo staff.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cassa con microfono</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cassa amplificata con microfono per le chiamate alle partenze.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Timer per partenza</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Timer per scandire le partenze.</t>
+  </si>
+  <si>
     <t xml:space="preserve">TOTALE BASE (voci «Nel totale» = Sì)</t>
   </si>
   <si>
@@ -410,6 +464,12 @@
   </si>
   <si>
     <t xml:space="preserve">Accoglienza e punto ristoro</t>
+  </si>
+  <si>
+    <t xml:space="preserve">E</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Organizzazione e staff</t>
   </si>
 </sst>
 </file>
@@ -1550,9 +1610,9 @@
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>'Riepilogo per area'!$B$5:$B$8</c:f>
+              <c:f>'Riepilogo per area'!$B$5:$B$9</c:f>
               <c:strCache>
-                <c:ptCount val="4"/>
+                <c:ptCount val="5"/>
                 <c:pt idx="0">
                   <c:v>Stampa e comunicazione</c:v>
                 </c:pt>
@@ -1565,15 +1625,18 @@
                 <c:pt idx="3">
                   <c:v>Accoglienza e punto ristoro</c:v>
                 </c:pt>
+                <c:pt idx="4">
+                  <c:v>Organizzazione e staff</c:v>
+                </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'Riepilogo per area'!$D$5:$D$8</c:f>
+              <c:f>'Riepilogo per area'!$D$5:$D$9</c:f>
               <c:numCache>
                 <c:formatCode>"€ "#,##0.00;"-€ "#,##0.00;\–</c:formatCode>
-                <c:ptCount val="4"/>
+                <c:ptCount val="5"/>
                 <c:pt idx="0">
                   <c:v>311.65</c:v>
                 </c:pt>
@@ -1584,7 +1647,10 @@
                   <c:v>1379</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>448</c:v>
+                  <c:v>518</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>150</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1592,11 +1658,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="94149724"/>
-        <c:axId val="81542354"/>
+        <c:axId val="86551681"/>
+        <c:axId val="45947816"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="94149724"/>
+        <c:axId val="86551681"/>
         <c:scaling>
           <c:orientation val="maxMin"/>
         </c:scaling>
@@ -1628,7 +1694,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="81542354"/>
+        <c:crossAx val="45947816"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1636,7 +1702,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="81542354"/>
+        <c:axId val="45947816"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1668,7 +1734,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="94149724"/>
+        <c:crossAx val="86551681"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1744,14 +1810,14 @@
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>11</xdr:row>
+      <xdr:row>12</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>5</xdr:col>
       <xdr:colOff>1122840</xdr:colOff>
-      <xdr:row>25</xdr:row>
-      <xdr:rowOff>32760</xdr:rowOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>32400</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -1759,7 +1825,7 @@
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
-        <a:off x="423000" y="2962440"/>
+        <a:off x="423000" y="3267000"/>
         <a:ext cx="6479640" cy="2699640"/>
       </xdr:xfrm>
       <a:graphic>
@@ -1954,7 +2020,7 @@
     <tabColor rgb="FF0072CE"/>
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:P37"/>
+  <dimension ref="A1:P43"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5"/>
@@ -2063,23 +2129,23 @@
     </row>
     <row r="6" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B6" s="7" t="n">
-        <f aca="false">SUMIFS($I$11:$I$30,$L$11:$L$30,"Sì")</f>
-        <v>3182.65</v>
+        <f aca="false">SUMIFS($I$11:$I$36,$L$11:$L$36,"Sì")</f>
+        <v>3402.65</v>
       </c>
       <c r="C6" s="7"/>
       <c r="D6" s="8" t="n">
-        <f aca="false">SUMIFS($I$11:$I$30,$K$11:$K$30,"Opzionale",$L$11:$L$30,"No")</f>
+        <f aca="false">SUMIFS($I$11:$I$36,$K$11:$K$36,"Opzionale",$L$11:$L$36,"No")</f>
         <v>2000</v>
       </c>
       <c r="E6" s="9" t="n">
         <f aca="false">B6+D6</f>
-        <v>5182.65</v>
+        <v>5402.65</v>
       </c>
       <c r="F6" s="9"/>
       <c r="G6" s="9"/>
       <c r="H6" s="10" t="n">
-        <f aca="false">COUNTIFS($K$11:$K$30,"Da definire")</f>
-        <v>4</v>
+        <f aca="false">COUNTIFS($K$11:$K$36,"Da definire")</f>
+        <v>6</v>
       </c>
       <c r="I6" s="10"/>
       <c r="J6" s="11"/>
@@ -2717,36 +2783,32 @@
         <v>13</v>
       </c>
       <c r="B23" s="18" t="s">
+        <v>66</v>
+      </c>
+      <c r="C23" s="19" t="s">
         <v>81</v>
       </c>
-      <c r="C23" s="19" t="s">
+      <c r="D23" s="20" t="s">
         <v>82</v>
       </c>
-      <c r="D23" s="20" t="s">
-        <v>83</v>
-      </c>
       <c r="E23" s="21"/>
-      <c r="F23" s="22" t="n">
-        <v>4</v>
-      </c>
+      <c r="F23" s="22"/>
       <c r="G23" s="23" t="s">
         <v>30</v>
       </c>
-      <c r="H23" s="24" t="n">
-        <v>37</v>
-      </c>
-      <c r="I23" s="25" t="n">
+      <c r="H23" s="24"/>
+      <c r="I23" s="25" t="str">
         <f aca="false">IF(OR(F23="",H23=""),"",F23*H23)</f>
-        <v>148</v>
+        <v/>
       </c>
       <c r="J23" s="23" t="s">
         <v>44</v>
       </c>
       <c r="K23" s="26" t="s">
-        <v>72</v>
+        <v>64</v>
       </c>
       <c r="L23" s="27" t="s">
-        <v>33</v>
+        <v>40</v>
       </c>
       <c r="M23" s="28" t="s">
         <v>34</v>
@@ -2756,7 +2818,7 @@
         <v>35</v>
       </c>
       <c r="P23" s="31" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2764,7 +2826,7 @@
         <v>14</v>
       </c>
       <c r="B24" s="33" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="C24" s="34" t="s">
         <v>85</v>
@@ -2779,16 +2841,18 @@
       <c r="G24" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="H24" s="24"/>
-      <c r="I24" s="37" t="str">
+      <c r="H24" s="24" t="n">
+        <v>37</v>
+      </c>
+      <c r="I24" s="37" t="n">
         <f aca="false">IF(OR(F24="",H24=""),"",F24*H24)</f>
-        <v/>
+        <v>148</v>
       </c>
       <c r="J24" s="36" t="s">
         <v>44</v>
       </c>
       <c r="K24" s="38" t="s">
-        <v>45</v>
+        <v>72</v>
       </c>
       <c r="L24" s="39" t="s">
         <v>33</v>
@@ -2809,7 +2873,7 @@
         <v>15</v>
       </c>
       <c r="B25" s="18" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="C25" s="19" t="s">
         <v>88</v>
@@ -2819,23 +2883,21 @@
       </c>
       <c r="E25" s="21"/>
       <c r="F25" s="22" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G25" s="23" t="s">
-        <v>90</v>
-      </c>
-      <c r="H25" s="24" t="n">
-        <v>300</v>
-      </c>
-      <c r="I25" s="25" t="n">
+        <v>30</v>
+      </c>
+      <c r="H25" s="24"/>
+      <c r="I25" s="25" t="str">
         <f aca="false">IF(OR(F25="",H25=""),"",F25*H25)</f>
-        <v>300</v>
+        <v/>
       </c>
       <c r="J25" s="23" t="s">
         <v>44</v>
       </c>
       <c r="K25" s="26" t="s">
-        <v>32</v>
+        <v>45</v>
       </c>
       <c r="L25" s="27" t="s">
         <v>33</v>
@@ -2847,27 +2909,49 @@
       <c r="O25" s="30" t="s">
         <v>35</v>
       </c>
-      <c r="P25" s="31"/>
+      <c r="P25" s="31" t="s">
+        <v>90</v>
+      </c>
     </row>
     <row r="26" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="32" t="n">
         <v>16</v>
       </c>
-      <c r="B26" s="33"/>
-      <c r="C26" s="34"/>
-      <c r="D26" s="35"/>
+      <c r="B26" s="33" t="s">
+        <v>84</v>
+      </c>
+      <c r="C26" s="34" t="s">
+        <v>91</v>
+      </c>
+      <c r="D26" s="35" t="s">
+        <v>92</v>
+      </c>
       <c r="E26" s="21"/>
-      <c r="F26" s="22"/>
-      <c r="G26" s="36"/>
-      <c r="H26" s="24"/>
-      <c r="I26" s="37" t="str">
+      <c r="F26" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="G26" s="36" t="s">
+        <v>93</v>
+      </c>
+      <c r="H26" s="24" t="n">
+        <v>300</v>
+      </c>
+      <c r="I26" s="37" t="n">
         <f aca="false">IF(OR(F26="",H26=""),"",F26*H26)</f>
-        <v/>
-      </c>
-      <c r="J26" s="36"/>
-      <c r="K26" s="38"/>
-      <c r="L26" s="39"/>
-      <c r="M26" s="40"/>
+        <v>300</v>
+      </c>
+      <c r="J26" s="36" t="s">
+        <v>44</v>
+      </c>
+      <c r="K26" s="38" t="s">
+        <v>32</v>
+      </c>
+      <c r="L26" s="39" t="s">
+        <v>33</v>
+      </c>
+      <c r="M26" s="40" t="s">
+        <v>34</v>
+      </c>
       <c r="N26" s="29"/>
       <c r="O26" s="30" t="s">
         <v>35</v>
@@ -2878,152 +2962,402 @@
       <c r="A27" s="17" t="n">
         <v>17</v>
       </c>
-      <c r="B27" s="18"/>
-      <c r="C27" s="19"/>
-      <c r="D27" s="20"/>
+      <c r="B27" s="18" t="s">
+        <v>84</v>
+      </c>
+      <c r="C27" s="19" t="s">
+        <v>94</v>
+      </c>
+      <c r="D27" s="20" t="s">
+        <v>95</v>
+      </c>
       <c r="E27" s="21"/>
-      <c r="F27" s="22"/>
-      <c r="G27" s="23"/>
-      <c r="H27" s="24"/>
-      <c r="I27" s="25" t="str">
+      <c r="F27" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="G27" s="23" t="s">
+        <v>54</v>
+      </c>
+      <c r="H27" s="24" t="n">
+        <v>70</v>
+      </c>
+      <c r="I27" s="25" t="n">
         <f aca="false">IF(OR(F27="",H27=""),"",F27*H27)</f>
-        <v/>
-      </c>
-      <c r="J27" s="23"/>
-      <c r="K27" s="26"/>
-      <c r="L27" s="27"/>
-      <c r="M27" s="28"/>
+        <v>70</v>
+      </c>
+      <c r="J27" s="23" t="s">
+        <v>44</v>
+      </c>
+      <c r="K27" s="26" t="s">
+        <v>32</v>
+      </c>
+      <c r="L27" s="27" t="s">
+        <v>33</v>
+      </c>
+      <c r="M27" s="28" t="s">
+        <v>34</v>
+      </c>
       <c r="N27" s="29"/>
       <c r="O27" s="30" t="s">
         <v>35</v>
       </c>
-      <c r="P27" s="31"/>
+      <c r="P27" s="31" t="s">
+        <v>96</v>
+      </c>
     </row>
     <row r="28" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="32" t="n">
         <v>18</v>
       </c>
-      <c r="B28" s="33"/>
-      <c r="C28" s="34"/>
-      <c r="D28" s="35"/>
+      <c r="B28" s="33" t="s">
+        <v>97</v>
+      </c>
+      <c r="C28" s="34" t="s">
+        <v>98</v>
+      </c>
+      <c r="D28" s="35" t="s">
+        <v>99</v>
+      </c>
       <c r="E28" s="21"/>
-      <c r="F28" s="22"/>
-      <c r="G28" s="36"/>
+      <c r="F28" s="22" t="n">
+        <v>10</v>
+      </c>
+      <c r="G28" s="36" t="s">
+        <v>30</v>
+      </c>
       <c r="H28" s="24"/>
       <c r="I28" s="37" t="str">
         <f aca="false">IF(OR(F28="",H28=""),"",F28*H28)</f>
         <v/>
       </c>
-      <c r="J28" s="36"/>
-      <c r="K28" s="38"/>
-      <c r="L28" s="39"/>
-      <c r="M28" s="40"/>
+      <c r="J28" s="36" t="s">
+        <v>44</v>
+      </c>
+      <c r="K28" s="38" t="s">
+        <v>45</v>
+      </c>
+      <c r="L28" s="39" t="s">
+        <v>33</v>
+      </c>
+      <c r="M28" s="40" t="s">
+        <v>34</v>
+      </c>
       <c r="N28" s="29"/>
       <c r="O28" s="30" t="s">
         <v>35</v>
       </c>
-      <c r="P28" s="41"/>
+      <c r="P28" s="41" t="s">
+        <v>100</v>
+      </c>
     </row>
     <row r="29" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="17" t="n">
         <v>19</v>
       </c>
-      <c r="B29" s="18"/>
-      <c r="C29" s="19"/>
-      <c r="D29" s="20"/>
+      <c r="B29" s="18" t="s">
+        <v>97</v>
+      </c>
+      <c r="C29" s="19" t="s">
+        <v>101</v>
+      </c>
+      <c r="D29" s="20" t="s">
+        <v>102</v>
+      </c>
       <c r="E29" s="21"/>
       <c r="F29" s="22"/>
-      <c r="G29" s="23"/>
+      <c r="G29" s="23" t="s">
+        <v>103</v>
+      </c>
       <c r="H29" s="24"/>
       <c r="I29" s="25" t="str">
         <f aca="false">IF(OR(F29="",H29=""),"",F29*H29)</f>
         <v/>
       </c>
-      <c r="J29" s="23"/>
-      <c r="K29" s="26"/>
-      <c r="L29" s="27"/>
-      <c r="M29" s="28"/>
+      <c r="J29" s="23" t="s">
+        <v>44</v>
+      </c>
+      <c r="K29" s="26" t="s">
+        <v>45</v>
+      </c>
+      <c r="L29" s="27" t="s">
+        <v>33</v>
+      </c>
+      <c r="M29" s="28" t="s">
+        <v>34</v>
+      </c>
       <c r="N29" s="29"/>
       <c r="O29" s="30" t="s">
         <v>35</v>
       </c>
-      <c r="P29" s="31"/>
+      <c r="P29" s="31" t="s">
+        <v>104</v>
+      </c>
     </row>
     <row r="30" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="32" t="n">
         <v>20</v>
       </c>
-      <c r="B30" s="33"/>
-      <c r="C30" s="34"/>
-      <c r="D30" s="35"/>
+      <c r="B30" s="33" t="s">
+        <v>97</v>
+      </c>
+      <c r="C30" s="34" t="s">
+        <v>105</v>
+      </c>
+      <c r="D30" s="35" t="s">
+        <v>106</v>
+      </c>
       <c r="E30" s="21"/>
-      <c r="F30" s="22"/>
-      <c r="G30" s="36"/>
-      <c r="H30" s="24"/>
-      <c r="I30" s="37" t="str">
+      <c r="F30" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="G30" s="36" t="s">
+        <v>30</v>
+      </c>
+      <c r="H30" s="24" t="n">
+        <v>70</v>
+      </c>
+      <c r="I30" s="37" t="n">
         <f aca="false">IF(OR(F30="",H30=""),"",F30*H30)</f>
-        <v/>
-      </c>
-      <c r="J30" s="36"/>
-      <c r="K30" s="38"/>
-      <c r="L30" s="39"/>
-      <c r="M30" s="40"/>
+        <v>70</v>
+      </c>
+      <c r="J30" s="36" t="s">
+        <v>44</v>
+      </c>
+      <c r="K30" s="38" t="s">
+        <v>32</v>
+      </c>
+      <c r="L30" s="39" t="s">
+        <v>33</v>
+      </c>
+      <c r="M30" s="40" t="s">
+        <v>34</v>
+      </c>
       <c r="N30" s="29"/>
       <c r="O30" s="30" t="s">
         <v>35</v>
       </c>
       <c r="P30" s="41"/>
     </row>
-    <row r="31" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="1"/>
-      <c r="B31" s="1"/>
-      <c r="C31" s="42" t="s">
-        <v>91</v>
-      </c>
-      <c r="D31" s="1"/>
-      <c r="E31" s="1"/>
-      <c r="F31" s="1"/>
-      <c r="G31" s="1"/>
-      <c r="H31" s="1"/>
-      <c r="I31" s="43" t="n">
-        <f aca="false">SUMIFS($I$11:$I$30,$L$11:$L$30,"Sì")</f>
-        <v>3182.65</v>
-      </c>
-      <c r="J31" s="1"/>
-      <c r="K31" s="1"/>
-      <c r="L31" s="1"/>
-      <c r="M31" s="1"/>
-      <c r="N31" s="1"/>
-      <c r="O31" s="1"/>
-      <c r="P31" s="1"/>
-    </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B33" s="44" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B34" s="45" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B35" s="45" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B36" s="45" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B37" s="45" t="s">
-        <v>96</v>
+    <row r="31" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="17" t="n">
+        <v>21</v>
+      </c>
+      <c r="B31" s="18" t="s">
+        <v>97</v>
+      </c>
+      <c r="C31" s="19" t="s">
+        <v>107</v>
+      </c>
+      <c r="D31" s="20" t="s">
+        <v>108</v>
+      </c>
+      <c r="E31" s="21"/>
+      <c r="F31" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="G31" s="23" t="s">
+        <v>30</v>
+      </c>
+      <c r="H31" s="24" t="n">
+        <v>80</v>
+      </c>
+      <c r="I31" s="25" t="n">
+        <f aca="false">IF(OR(F31="",H31=""),"",F31*H31)</f>
+        <v>80</v>
+      </c>
+      <c r="J31" s="23" t="s">
+        <v>44</v>
+      </c>
+      <c r="K31" s="26" t="s">
+        <v>32</v>
+      </c>
+      <c r="L31" s="27" t="s">
+        <v>33</v>
+      </c>
+      <c r="M31" s="28" t="s">
+        <v>34</v>
+      </c>
+      <c r="N31" s="29"/>
+      <c r="O31" s="30" t="s">
+        <v>35</v>
+      </c>
+      <c r="P31" s="31"/>
+    </row>
+    <row r="32" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="32" t="n">
+        <v>22</v>
+      </c>
+      <c r="B32" s="33"/>
+      <c r="C32" s="34"/>
+      <c r="D32" s="35"/>
+      <c r="E32" s="21"/>
+      <c r="F32" s="22"/>
+      <c r="G32" s="36"/>
+      <c r="H32" s="24"/>
+      <c r="I32" s="37" t="str">
+        <f aca="false">IF(OR(F32="",H32=""),"",F32*H32)</f>
+        <v/>
+      </c>
+      <c r="J32" s="36"/>
+      <c r="K32" s="38"/>
+      <c r="L32" s="39"/>
+      <c r="M32" s="40"/>
+      <c r="N32" s="29"/>
+      <c r="O32" s="30" t="s">
+        <v>35</v>
+      </c>
+      <c r="P32" s="41"/>
+    </row>
+    <row r="33" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="17" t="n">
+        <v>23</v>
+      </c>
+      <c r="B33" s="18"/>
+      <c r="C33" s="19"/>
+      <c r="D33" s="20"/>
+      <c r="E33" s="21"/>
+      <c r="F33" s="22"/>
+      <c r="G33" s="23"/>
+      <c r="H33" s="24"/>
+      <c r="I33" s="25" t="str">
+        <f aca="false">IF(OR(F33="",H33=""),"",F33*H33)</f>
+        <v/>
+      </c>
+      <c r="J33" s="23"/>
+      <c r="K33" s="26"/>
+      <c r="L33" s="27"/>
+      <c r="M33" s="28"/>
+      <c r="N33" s="29"/>
+      <c r="O33" s="30" t="s">
+        <v>35</v>
+      </c>
+      <c r="P33" s="31"/>
+    </row>
+    <row r="34" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="32" t="n">
+        <v>24</v>
+      </c>
+      <c r="B34" s="33"/>
+      <c r="C34" s="34"/>
+      <c r="D34" s="35"/>
+      <c r="E34" s="21"/>
+      <c r="F34" s="22"/>
+      <c r="G34" s="36"/>
+      <c r="H34" s="24"/>
+      <c r="I34" s="37" t="str">
+        <f aca="false">IF(OR(F34="",H34=""),"",F34*H34)</f>
+        <v/>
+      </c>
+      <c r="J34" s="36"/>
+      <c r="K34" s="38"/>
+      <c r="L34" s="39"/>
+      <c r="M34" s="40"/>
+      <c r="N34" s="29"/>
+      <c r="O34" s="30" t="s">
+        <v>35</v>
+      </c>
+      <c r="P34" s="41"/>
+    </row>
+    <row r="35" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A35" s="17" t="n">
+        <v>25</v>
+      </c>
+      <c r="B35" s="18"/>
+      <c r="C35" s="19"/>
+      <c r="D35" s="20"/>
+      <c r="E35" s="21"/>
+      <c r="F35" s="22"/>
+      <c r="G35" s="23"/>
+      <c r="H35" s="24"/>
+      <c r="I35" s="25" t="str">
+        <f aca="false">IF(OR(F35="",H35=""),"",F35*H35)</f>
+        <v/>
+      </c>
+      <c r="J35" s="23"/>
+      <c r="K35" s="26"/>
+      <c r="L35" s="27"/>
+      <c r="M35" s="28"/>
+      <c r="N35" s="29"/>
+      <c r="O35" s="30" t="s">
+        <v>35</v>
+      </c>
+      <c r="P35" s="31"/>
+    </row>
+    <row r="36" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A36" s="32" t="n">
+        <v>26</v>
+      </c>
+      <c r="B36" s="33"/>
+      <c r="C36" s="34"/>
+      <c r="D36" s="35"/>
+      <c r="E36" s="21"/>
+      <c r="F36" s="22"/>
+      <c r="G36" s="36"/>
+      <c r="H36" s="24"/>
+      <c r="I36" s="37" t="str">
+        <f aca="false">IF(OR(F36="",H36=""),"",F36*H36)</f>
+        <v/>
+      </c>
+      <c r="J36" s="36"/>
+      <c r="K36" s="38"/>
+      <c r="L36" s="39"/>
+      <c r="M36" s="40"/>
+      <c r="N36" s="29"/>
+      <c r="O36" s="30" t="s">
+        <v>35</v>
+      </c>
+      <c r="P36" s="41"/>
+    </row>
+    <row r="37" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A37" s="1"/>
+      <c r="B37" s="1"/>
+      <c r="C37" s="42" t="s">
+        <v>109</v>
+      </c>
+      <c r="D37" s="1"/>
+      <c r="E37" s="1"/>
+      <c r="F37" s="1"/>
+      <c r="G37" s="1"/>
+      <c r="H37" s="1"/>
+      <c r="I37" s="43" t="n">
+        <f aca="false">SUMIFS($I$11:$I$36,$L$11:$L$36,"Sì")</f>
+        <v>3402.65</v>
+      </c>
+      <c r="J37" s="1"/>
+      <c r="K37" s="1"/>
+      <c r="L37" s="1"/>
+      <c r="M37" s="1"/>
+      <c r="N37" s="1"/>
+      <c r="O37" s="1"/>
+      <c r="P37" s="1"/>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B39" s="44" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B40" s="45" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B41" s="45" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B42" s="45" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B43" s="45" t="s">
+        <v>114</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A10:P30"/>
+  <autoFilter ref="A10:P36"/>
   <mergeCells count="10">
     <mergeCell ref="B5:C5"/>
     <mergeCell ref="E5:G5"/>
@@ -3036,7 +3370,7 @@
     <mergeCell ref="J6:L6"/>
     <mergeCell ref="M6:N6"/>
   </mergeCells>
-  <conditionalFormatting sqref="K11:K30">
+  <conditionalFormatting sqref="K11:K36">
     <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="19">
       <formula>$K11="Preventivo"</formula>
     </cfRule>
@@ -3053,7 +3387,7 @@
       <formula>$K11="Da definire"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="M11:M30">
+  <conditionalFormatting sqref="M11:M36">
     <cfRule type="expression" priority="7" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="24">
       <formula>$M11="Ordinato"</formula>
     </cfRule>
@@ -3064,21 +3398,21 @@
       <formula>$M11="Pagato"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I11:I30">
+  <conditionalFormatting sqref="I11:I36">
     <cfRule type="expression" priority="10" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="27">
       <formula>$L11="No"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="3">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="K11:K30" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="K11:K36" type="list">
       <formula1>"Preventivo,Stima,Opzionale,Alternativa,Da definire"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="L11:L30" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="L11:L36" type="list">
       <formula1>"Sì,No"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="M11:M30" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="M11:M36" type="list">
       <formula1>"Da ordinare,Ordinato,Consegnato,Pagato"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -3105,7 +3439,7 @@
     <tabColor rgb="FF0A0C0A"/>
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G9"/>
+  <dimension ref="A1:G10"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="6"/>
@@ -3118,7 +3452,7 @@
     <row r="1" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1"/>
       <c r="B1" s="46" t="s">
-        <v>97</v>
+        <v>115</v>
       </c>
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
@@ -3129,7 +3463,7 @@
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1"/>
       <c r="B2" s="47" t="s">
-        <v>98</v>
+        <v>116</v>
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
@@ -3143,7 +3477,7 @@
         <v>12</v>
       </c>
       <c r="C4" s="48" t="s">
-        <v>99</v>
+        <v>117</v>
       </c>
       <c r="D4" s="48" t="s">
         <v>3</v>
@@ -3155,26 +3489,26 @@
         <v>19</v>
       </c>
       <c r="G4" s="48" t="s">
-        <v>100</v>
+        <v>118</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="50" t="s">
-        <v>101</v>
+        <v>119</v>
       </c>
       <c r="B5" s="51" t="s">
-        <v>102</v>
+        <v>120</v>
       </c>
       <c r="C5" s="52" t="n">
-        <f aca="false">COUNTIFS('Piano di spesa'!$B$11:$B$30,"A · Stampa e comunicazione")</f>
+        <f aca="false">COUNTIFS('Piano di spesa'!$B$11:$B$36,"A · Stampa e comunicazione")</f>
         <v>4</v>
       </c>
       <c r="D5" s="53" t="n">
-        <f aca="false">SUMIFS('Piano di spesa'!$I$11:$I$30,'Piano di spesa'!$B$11:$B$30,"A · Stampa e comunicazione",'Piano di spesa'!$L$11:$L$30,"Sì")</f>
+        <f aca="false">SUMIFS('Piano di spesa'!$I$11:$I$36,'Piano di spesa'!$B$11:$B$36,"A · Stampa e comunicazione",'Piano di spesa'!$L$11:$L$36,"Sì")</f>
         <v>311.65</v>
       </c>
       <c r="E5" s="54" t="n">
-        <f aca="false">SUMIFS('Piano di spesa'!$I$11:$I$30,'Piano di spesa'!$B$11:$B$30,"A · Stampa e comunicazione",'Piano di spesa'!$K$11:$K$30,"Opzionale",'Piano di spesa'!$L$11:$L$30,"No")</f>
+        <f aca="false">SUMIFS('Piano di spesa'!$I$11:$I$36,'Piano di spesa'!$B$11:$B$36,"A · Stampa e comunicazione",'Piano di spesa'!$K$11:$K$36,"Opzionale",'Piano di spesa'!$L$11:$L$36,"No")</f>
         <v>0</v>
       </c>
       <c r="F5" s="54" t="n">
@@ -3182,27 +3516,27 @@
         <v>311.65</v>
       </c>
       <c r="G5" s="55" t="n">
-        <f aca="false">IF($D$9=0,0,D5/$D$9)</f>
-        <v>0.0979215433679481</v>
+        <f aca="false">IF($D$10=0,0,D5/$D$10)</f>
+        <v>0.091590378087667</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="50" t="s">
-        <v>103</v>
+        <v>121</v>
       </c>
       <c r="B6" s="51" t="s">
-        <v>104</v>
+        <v>122</v>
       </c>
       <c r="C6" s="52" t="n">
-        <f aca="false">COUNTIFS('Piano di spesa'!$B$11:$B$30,"B · Allestimento del campo")</f>
+        <f aca="false">COUNTIFS('Piano di spesa'!$B$11:$B$36,"B · Allestimento del campo")</f>
         <v>4</v>
       </c>
       <c r="D6" s="53" t="n">
-        <f aca="false">SUMIFS('Piano di spesa'!$I$11:$I$30,'Piano di spesa'!$B$11:$B$30,"B · Allestimento del campo",'Piano di spesa'!$L$11:$L$30,"Sì")</f>
+        <f aca="false">SUMIFS('Piano di spesa'!$I$11:$I$36,'Piano di spesa'!$B$11:$B$36,"B · Allestimento del campo",'Piano di spesa'!$L$11:$L$36,"Sì")</f>
         <v>1044</v>
       </c>
       <c r="E6" s="54" t="n">
-        <f aca="false">SUMIFS('Piano di spesa'!$I$11:$I$30,'Piano di spesa'!$B$11:$B$30,"B · Allestimento del campo",'Piano di spesa'!$K$11:$K$30,"Opzionale",'Piano di spesa'!$L$11:$L$30,"No")</f>
+        <f aca="false">SUMIFS('Piano di spesa'!$I$11:$I$36,'Piano di spesa'!$B$11:$B$36,"B · Allestimento del campo",'Piano di spesa'!$K$11:$K$36,"Opzionale",'Piano di spesa'!$L$11:$L$36,"No")</f>
         <v>2000</v>
       </c>
       <c r="F6" s="54" t="n">
@@ -3210,27 +3544,27 @@
         <v>3044</v>
       </c>
       <c r="G6" s="55" t="n">
-        <f aca="false">IF($D$9=0,0,D6/$D$9)</f>
-        <v>0.328028529684383</v>
+        <f aca="false">IF($D$10=0,0,D6/$D$10)</f>
+        <v>0.306819684657546</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="50" t="s">
-        <v>105</v>
+        <v>123</v>
       </c>
       <c r="B7" s="51" t="s">
-        <v>106</v>
+        <v>124</v>
       </c>
       <c r="C7" s="52" t="n">
-        <f aca="false">COUNTIFS('Piano di spesa'!$B$11:$B$30,"C · Immagine, media e presentazione")</f>
-        <v>4</v>
+        <f aca="false">COUNTIFS('Piano di spesa'!$B$11:$B$36,"C · Immagine, media e presentazione")</f>
+        <v>5</v>
       </c>
       <c r="D7" s="53" t="n">
-        <f aca="false">SUMIFS('Piano di spesa'!$I$11:$I$30,'Piano di spesa'!$B$11:$B$30,"C · Immagine, media e presentazione",'Piano di spesa'!$L$11:$L$30,"Sì")</f>
+        <f aca="false">SUMIFS('Piano di spesa'!$I$11:$I$36,'Piano di spesa'!$B$11:$B$36,"C · Immagine, media e presentazione",'Piano di spesa'!$L$11:$L$36,"Sì")</f>
         <v>1379</v>
       </c>
       <c r="E7" s="54" t="n">
-        <f aca="false">SUMIFS('Piano di spesa'!$I$11:$I$30,'Piano di spesa'!$B$11:$B$30,"C · Immagine, media e presentazione",'Piano di spesa'!$K$11:$K$30,"Opzionale",'Piano di spesa'!$L$11:$L$30,"No")</f>
+        <f aca="false">SUMIFS('Piano di spesa'!$I$11:$I$36,'Piano di spesa'!$B$11:$B$36,"C · Immagine, media e presentazione",'Piano di spesa'!$K$11:$K$36,"Opzionale",'Piano di spesa'!$L$11:$L$36,"No")</f>
         <v>0</v>
       </c>
       <c r="F7" s="54" t="n">
@@ -3238,61 +3572,89 @@
         <v>1379</v>
       </c>
       <c r="G7" s="55" t="n">
-        <f aca="false">IF($D$9=0,0,D7/$D$9)</f>
-        <v>0.43328672647008</v>
+        <f aca="false">IF($D$10=0,0,D7/$D$10)</f>
+        <v>0.405272361247851</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="50" t="s">
-        <v>107</v>
+        <v>125</v>
       </c>
       <c r="B8" s="51" t="s">
-        <v>108</v>
+        <v>126</v>
       </c>
       <c r="C8" s="52" t="n">
-        <f aca="false">COUNTIFS('Piano di spesa'!$B$11:$B$30,"D · Accoglienza e punto ristoro")</f>
-        <v>3</v>
+        <f aca="false">COUNTIFS('Piano di spesa'!$B$11:$B$36,"D · Accoglienza e punto ristoro")</f>
+        <v>4</v>
       </c>
       <c r="D8" s="53" t="n">
-        <f aca="false">SUMIFS('Piano di spesa'!$I$11:$I$30,'Piano di spesa'!$B$11:$B$30,"D · Accoglienza e punto ristoro",'Piano di spesa'!$L$11:$L$30,"Sì")</f>
-        <v>448</v>
+        <f aca="false">SUMIFS('Piano di spesa'!$I$11:$I$36,'Piano di spesa'!$B$11:$B$36,"D · Accoglienza e punto ristoro",'Piano di spesa'!$L$11:$L$36,"Sì")</f>
+        <v>518</v>
       </c>
       <c r="E8" s="54" t="n">
-        <f aca="false">SUMIFS('Piano di spesa'!$I$11:$I$30,'Piano di spesa'!$B$11:$B$30,"D · Accoglienza e punto ristoro",'Piano di spesa'!$K$11:$K$30,"Opzionale",'Piano di spesa'!$L$11:$L$30,"No")</f>
+        <f aca="false">SUMIFS('Piano di spesa'!$I$11:$I$36,'Piano di spesa'!$B$11:$B$36,"D · Accoglienza e punto ristoro",'Piano di spesa'!$K$11:$K$36,"Opzionale",'Piano di spesa'!$L$11:$L$36,"No")</f>
         <v>0</v>
       </c>
       <c r="F8" s="54" t="n">
         <f aca="false">D8+E8</f>
-        <v>448</v>
+        <v>518</v>
       </c>
       <c r="G8" s="55" t="n">
-        <f aca="false">IF($D$9=0,0,D8/$D$9)</f>
-        <v>0.140763200477589</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="1"/>
-      <c r="B9" s="56" t="s">
+        <f aca="false">IF($D$10=0,0,D8/$D$10)</f>
+        <v>0.152234287981426</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="50" t="s">
+        <v>127</v>
+      </c>
+      <c r="B9" s="51" t="s">
+        <v>128</v>
+      </c>
+      <c r="C9" s="52" t="n">
+        <f aca="false">COUNTIFS('Piano di spesa'!$B$11:$B$36,"E · Organizzazione e staff")</f>
+        <v>4</v>
+      </c>
+      <c r="D9" s="53" t="n">
+        <f aca="false">SUMIFS('Piano di spesa'!$I$11:$I$36,'Piano di spesa'!$B$11:$B$36,"E · Organizzazione e staff",'Piano di spesa'!$L$11:$L$36,"Sì")</f>
+        <v>150</v>
+      </c>
+      <c r="E9" s="54" t="n">
+        <f aca="false">SUMIFS('Piano di spesa'!$I$11:$I$36,'Piano di spesa'!$B$11:$B$36,"E · Organizzazione e staff",'Piano di spesa'!$K$11:$K$36,"Opzionale",'Piano di spesa'!$L$11:$L$36,"No")</f>
+        <v>0</v>
+      </c>
+      <c r="F9" s="54" t="n">
+        <f aca="false">D9+E9</f>
+        <v>150</v>
+      </c>
+      <c r="G9" s="55" t="n">
+        <f aca="false">IF($D$10=0,0,D9/$D$10)</f>
+        <v>0.0440832880255095</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="1"/>
+      <c r="B10" s="56" t="s">
         <v>19</v>
       </c>
-      <c r="C9" s="57" t="n">
-        <f aca="false">SUM(C5:C8)</f>
-        <v>15</v>
-      </c>
-      <c r="D9" s="58" t="n">
-        <f aca="false">SUM(D5:D8)</f>
-        <v>3182.65</v>
-      </c>
-      <c r="E9" s="59" t="n">
-        <f aca="false">SUM(E5:E8)</f>
+      <c r="C10" s="57" t="n">
+        <f aca="false">SUM(C5:C9)</f>
+        <v>21</v>
+      </c>
+      <c r="D10" s="58" t="n">
+        <f aca="false">SUM(D5:D9)</f>
+        <v>3402.65</v>
+      </c>
+      <c r="E10" s="59" t="n">
+        <f aca="false">SUM(E5:E9)</f>
         <v>2000</v>
       </c>
-      <c r="F9" s="59" t="n">
-        <f aca="false">SUM(F5:F8)</f>
-        <v>5182.65</v>
-      </c>
-      <c r="G9" s="60" t="n">
-        <f aca="false">IF($D$9=0,0,SUM(G5:G8))</f>
+      <c r="F10" s="59" t="n">
+        <f aca="false">SUM(F5:F9)</f>
+        <v>5402.65</v>
+      </c>
+      <c r="G10" s="60" t="n">
+        <f aca="false">IF($D$10=0,0,SUM(G5:G9))</f>
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Piano di spesa Tappa Zero: nuovi preventivi, collarini e cubi
- Brochure 63 × 29,7 cm, 100 pz, € 180 al posto del pieghevole A4; A3 resta
  come alternativa.
- Pannelli buca forex 125 × 45 con supporto in polionda, 18 × € 54 + IVA.
- Partenze Donne in Bi-Bond, 13 × € 4 + IVA; Junior ancora da quotare.
- Wall: banner con asola 210 × 160/170, € 85 + IVA.
- Sedie per gazebo: 10 × € 70.
- Nuove voci: cubi in polionda 30 × 30 (€ 150), collarini con doppio
  moschettone (100 pz, € 370). Totale base € 4.537.
- Scheda voce più compatta per tenere cinque voci in una pagina.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014EyPNYo6uPPTyzbFJvdbw6
</commit_message>
<xml_diff>
--- a/piano-spesa-tappa-zero-2026/dist/piano-spesa-tappa-zero-2026.xlsx
+++ b/piano-spesa-tappa-zero-2026/dist/piano-spesa-tappa-zero-2026.xlsx
@@ -13,7 +13,7 @@
   </sheets>
   <definedNames>
     <definedName function="false" hidden="false" localSheetId="0" name="_xlnm.Print_Titles" vbProcedure="false">'Piano di spesa'!$10:$10</definedName>
-    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">'Piano di spesa'!$A$10:$P$36</definedName>
+    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">'Piano di spesa'!$A$10:$P$38</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -38,7 +38,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Dal preventivo: € 71,65 complessivi per 250 pz,</t>
+          <t xml:space="preserve">Dal preventivo: € 180,00 complessivi per 100 pz,</t>
         </r>
       </text>
     </comment>
@@ -54,7 +54,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="H16" authorId="0">
+    <comment ref="H19" authorId="0">
       <text>
         <r>
           <rPr>
@@ -62,7 +62,19 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Dal preventivo: € 654,00 complessivi per 18 pz,</t>
+          <t xml:space="preserve">Dal preventivo: € 150,00 complessivi per 1 fornitura,</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="H33" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Dal preventivo: € 370,00 complessivi per 100 pz,</t>
         </r>
       </text>
     </comment>
@@ -83,7 +95,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="267" uniqueCount="129">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="287" uniqueCount="136">
   <si>
     <t xml:space="preserve">PIANO DI SPESA · TAPPA ZERO</t>
   </si>
@@ -169,46 +181,49 @@
     <t xml:space="preserve">A · Stampa e comunicazione</t>
   </si>
   <si>
-    <t xml:space="preserve">Pieghevole A4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2 pieghe, 6 facciate, formato A4 (21 × 29,7 cm) orizzontale.</t>
+    <t xml:space="preserve">Brochure pieghevole</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Formato aperto 63 × 29,7 cm: A4 a 2 pieghe, 6 facciate.</t>
   </si>
   <si>
     <t xml:space="preserve">pz</t>
   </si>
   <si>
+    <t xml:space="preserve">Da verificare</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Preventivo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sì</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Da ordinare</t>
+  </si>
+  <si>
+    <t xml:space="preserve">incolla qui la foto</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Preventivo precedente: 250 pz A4 a € 71,65 IVA inclusa.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pieghevole A3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2 pieghe, 6 facciate, formato A3 (29 × 42 cm) orizzontale.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Inclusa</t>
   </si>
   <si>
-    <t xml:space="preserve">Preventivo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sì</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Da ordinare</t>
-  </si>
-  <si>
-    <t xml:space="preserve">incolla qui la foto</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Prezzo complessivo per 250 pezzi, IVA compresa.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pieghevole A3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2 pieghe, 6 facciate, formato A3 (29 × 42 cm) orizzontale.</t>
-  </si>
-  <si>
     <t xml:space="preserve">Alternativa</t>
   </si>
   <si>
     <t xml:space="preserve">No</t>
   </si>
   <si>
-    <t xml:space="preserve">In alternativa al pieghevole A4 (n. 1): +€ 54,25 se si sceglie l'A3.</t>
+    <t xml:space="preserve">In alternativa alla brochure (n. 1): 250 pz A3 a € 125,90 IVA inclusa.</t>
   </si>
   <si>
     <t xml:space="preserve">Flyer promozioni</t>
@@ -217,9 +232,6 @@
     <t xml:space="preserve">Flyer con le promozioni della stagione da distribuire in tappa.</t>
   </si>
   <si>
-    <t xml:space="preserve">Da verificare</t>
-  </si>
-  <si>
     <t xml:space="preserve">Da definire</t>
   </si>
   <si>
@@ -253,22 +265,25 @@
     <t xml:space="preserve">Verificare il numero di bandiere compreso nella fornitura.</t>
   </si>
   <si>
-    <t xml:space="preserve">Pannelli forex presentazione buca</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Forex 70 × 100 cm con vernice protettiva antigraffio, uno per buca.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">€ 654 per i 18 pezzi.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Partenze forex Women e Junior</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Segnaletica in forex per le partenze dedicate Women e Junior.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Quantità e prezzo da definire.</t>
+    <t xml:space="preserve">Pannelli presentazione buca</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forex 5 mm personalizzato con supporto in polionda 5 mm, 125 × 45 cm, uno per buca.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Esclusa</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Preventivo precedente: forex 70 × 100 cm antigraffio, € 654 per 18 pezzi.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Partenze Donne</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cartello di partenza 21 × 15 cm con punta, in Bi-Bond.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Le partenze Junior sono ancora da quotare.</t>
   </si>
   <si>
     <t xml:space="preserve">Mini vele di partenza</t>
@@ -283,13 +298,25 @@
     <t xml:space="preserve">Voce eventuale: fuori dal totale base.</t>
   </si>
   <si>
+    <t xml:space="preserve">Cubi in polionda</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cubi in polionda 5 mm, 30 × 30 cm.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Verificare quanti cubi comprende la fornitura.</t>
+  </si>
+  <si>
     <t xml:space="preserve">C · Immagine, media e presentazione</t>
   </si>
   <si>
     <t xml:space="preserve">Wall per foto giocatori</t>
   </si>
   <si>
-    <t xml:space="preserve">Fondale pubblicitario 300 × 240 cm per le foto dei giocatori.</t>
+    <t xml:space="preserve">Banner con asola 210 × 160/170 cm per le foto dei giocatori.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Preventivo precedente: fondale 300 × 240 cm a € 579.</t>
   </si>
   <si>
     <t xml:space="preserve">Telo per videoproiettore</t>
@@ -373,7 +400,7 @@
     <t xml:space="preserve">Sedie per i gazebo dell'accoglienza e della segreteria.</t>
   </si>
   <si>
-    <t xml:space="preserve">Verificare quante sedie comprende la fornitura.</t>
+    <t xml:space="preserve">€ 70 a sedia.</t>
   </si>
   <si>
     <t xml:space="preserve">E · Organizzazione e staff</t>
@@ -412,19 +439,25 @@
     <t xml:space="preserve">Timer per scandire le partenze.</t>
   </si>
   <si>
+    <t xml:space="preserve">Collarini personalizzati</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Collarini con doppio moschettone, personalizzati.</t>
+  </si>
+  <si>
     <t xml:space="preserve">TOTALE BASE (voci «Nel totale» = Sì)</t>
   </si>
   <si>
     <t xml:space="preserve">Note</t>
   </si>
   <si>
-    <t xml:space="preserve">• Pieghevole A4 (n. 1) e A3 (n. 2) sono alternativi: nel totale base c'è l'A4. Per passare all'A3 invertire «Nel totale» sulle due righe.</t>
+    <t xml:space="preserve">• Brochure (n. 1) e pieghevole A3 (n. 2) sono alternativi: nel totale base c'è la brochure. Per passare all'A3 invertire «Nel totale» sulle due righe.</t>
   </si>
   <si>
     <t xml:space="preserve">• Mini vele (n. 8) è voce eventuale, fuori dal totale base. Telo proiettore (€ 80–100) e drone (€ 400–700): messo il massimo per prudenza.</t>
   </si>
   <si>
-    <t xml:space="preserve">• Tavoli ristoro: quantità 4 ipotizzata, da confermare. IVA indicata come inclusa solo dove il preventivo lo dice esplicitamente.</t>
+    <t xml:space="preserve">• Tavoli ristoro: quantità 4 ipotizzata, da confermare. IVA «Esclusa» o «Inclusa» solo dove il preventivo lo dice: altrimenti da verificare.</t>
   </si>
   <si>
     <t xml:space="preserve">• Foto: in Excel 365 selezionare la cella gialla → Inserisci → Immagini → Inserisci nella cella. Le righe libere in fondo sono pronte per nuove voci.</t>
@@ -1638,19 +1671,19 @@
                 <c:formatCode>"€ "#,##0.00;"-€ "#,##0.00;\–</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>311.65</c:v>
+                  <c:v>420</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>1044</c:v>
+                  <c:v>1564</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1379</c:v>
+                  <c:v>885</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>518</c:v>
+                  <c:v>1148</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>150</c:v>
+                  <c:v>520</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1658,11 +1691,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="86551681"/>
-        <c:axId val="45947816"/>
+        <c:axId val="67172425"/>
+        <c:axId val="23899440"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="86551681"/>
+        <c:axId val="67172425"/>
         <c:scaling>
           <c:orientation val="maxMin"/>
         </c:scaling>
@@ -1694,7 +1727,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="45947816"/>
+        <c:crossAx val="23899440"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1702,7 +1735,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="45947816"/>
+        <c:axId val="23899440"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1734,7 +1767,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="86551681"/>
+        <c:crossAx val="67172425"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2020,7 +2053,7 @@
     <tabColor rgb="FF0072CE"/>
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:P43"/>
+  <dimension ref="A1:P45"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5"/>
@@ -2129,23 +2162,23 @@
     </row>
     <row r="6" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B6" s="7" t="n">
-        <f aca="false">SUMIFS($I$11:$I$36,$L$11:$L$36,"Sì")</f>
-        <v>3402.65</v>
+        <f aca="false">SUMIFS($I$11:$I$38,$L$11:$L$38,"Sì")</f>
+        <v>4537</v>
       </c>
       <c r="C6" s="7"/>
       <c r="D6" s="8" t="n">
-        <f aca="false">SUMIFS($I$11:$I$36,$K$11:$K$36,"Opzionale",$L$11:$L$36,"No")</f>
+        <f aca="false">SUMIFS($I$11:$I$38,$K$11:$K$38,"Opzionale",$L$11:$L$38,"No")</f>
         <v>2000</v>
       </c>
       <c r="E6" s="9" t="n">
         <f aca="false">B6+D6</f>
-        <v>5402.65</v>
+        <v>6537</v>
       </c>
       <c r="F6" s="9"/>
       <c r="G6" s="9"/>
       <c r="H6" s="10" t="n">
-        <f aca="false">COUNTIFS($K$11:$K$36,"Da definire")</f>
-        <v>6</v>
+        <f aca="false">COUNTIFS($K$11:$K$38,"Da definire")</f>
+        <v>5</v>
       </c>
       <c r="I6" s="10"/>
       <c r="J6" s="11"/>
@@ -2230,18 +2263,18 @@
       </c>
       <c r="E11" s="21"/>
       <c r="F11" s="22" t="n">
-        <v>250</v>
+        <v>100</v>
       </c>
       <c r="G11" s="23" t="s">
         <v>30</v>
       </c>
       <c r="H11" s="24" t="n">
-        <f aca="false">71.65/250</f>
-        <v>0.2866</v>
+        <f aca="false">180/100</f>
+        <v>1.8</v>
       </c>
       <c r="I11" s="25" t="n">
         <f aca="false">IF(OR(F11="",H11=""),"",F11*H11)</f>
-        <v>71.65</v>
+        <v>180</v>
       </c>
       <c r="J11" s="23" t="s">
         <v>31</v>
@@ -2292,13 +2325,13 @@
         <v>125.9</v>
       </c>
       <c r="J12" s="36" t="s">
-        <v>31</v>
+        <v>39</v>
       </c>
       <c r="K12" s="38" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="L12" s="39" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="M12" s="40" t="s">
         <v>34</v>
@@ -2308,7 +2341,7 @@
         <v>35</v>
       </c>
       <c r="P12" s="41" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2319,10 +2352,10 @@
         <v>27</v>
       </c>
       <c r="C13" s="19" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D13" s="20" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="E13" s="21"/>
       <c r="F13" s="22"/>
@@ -2335,7 +2368,7 @@
         <v/>
       </c>
       <c r="J13" s="23" t="s">
-        <v>44</v>
+        <v>31</v>
       </c>
       <c r="K13" s="26" t="s">
         <v>45</v>
@@ -2382,7 +2415,7 @@
         <v>240</v>
       </c>
       <c r="J14" s="36" t="s">
-        <v>44</v>
+        <v>31</v>
       </c>
       <c r="K14" s="38" t="s">
         <v>32</v>
@@ -2431,7 +2464,7 @@
         <v>390</v>
       </c>
       <c r="J15" s="23" t="s">
-        <v>44</v>
+        <v>31</v>
       </c>
       <c r="K15" s="26" t="s">
         <v>32</v>
@@ -2473,15 +2506,14 @@
         <v>30</v>
       </c>
       <c r="H16" s="24" t="n">
-        <f aca="false">654/18</f>
-        <v>36.3333333333333</v>
+        <v>54</v>
       </c>
       <c r="I16" s="37" t="n">
         <f aca="false">IF(OR(F16="",H16=""),"",F16*H16)</f>
-        <v>654</v>
+        <v>972</v>
       </c>
       <c r="J16" s="36" t="s">
-        <v>44</v>
+        <v>58</v>
       </c>
       <c r="K16" s="38" t="s">
         <v>32</v>
@@ -2497,7 +2529,7 @@
         <v>35</v>
       </c>
       <c r="P16" s="41" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2508,26 +2540,30 @@
         <v>50</v>
       </c>
       <c r="C17" s="19" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D17" s="20" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="E17" s="21"/>
-      <c r="F17" s="22"/>
+      <c r="F17" s="22" t="n">
+        <v>13</v>
+      </c>
       <c r="G17" s="23" t="s">
         <v>30</v>
       </c>
-      <c r="H17" s="24"/>
-      <c r="I17" s="25" t="str">
+      <c r="H17" s="24" t="n">
+        <v>4</v>
+      </c>
+      <c r="I17" s="25" t="n">
         <f aca="false">IF(OR(F17="",H17=""),"",F17*H17)</f>
-        <v/>
+        <v>52</v>
       </c>
       <c r="J17" s="23" t="s">
-        <v>44</v>
+        <v>58</v>
       </c>
       <c r="K17" s="26" t="s">
-        <v>45</v>
+        <v>32</v>
       </c>
       <c r="L17" s="27" t="s">
         <v>33</v>
@@ -2540,7 +2576,7 @@
         <v>35</v>
       </c>
       <c r="P17" s="31" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2551,10 +2587,10 @@
         <v>50</v>
       </c>
       <c r="C18" s="34" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D18" s="35" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="E18" s="21"/>
       <c r="F18" s="22" t="n">
@@ -2571,13 +2607,13 @@
         <v>2000</v>
       </c>
       <c r="J18" s="36" t="s">
-        <v>44</v>
+        <v>31</v>
       </c>
       <c r="K18" s="38" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="L18" s="39" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="M18" s="40" t="s">
         <v>34</v>
@@ -2587,7 +2623,7 @@
         <v>35</v>
       </c>
       <c r="P18" s="41" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2595,7 +2631,7 @@
         <v>9</v>
       </c>
       <c r="B19" s="18" t="s">
-        <v>66</v>
+        <v>50</v>
       </c>
       <c r="C19" s="19" t="s">
         <v>67</v>
@@ -2608,17 +2644,18 @@
         <v>1</v>
       </c>
       <c r="G19" s="23" t="s">
-        <v>30</v>
+        <v>54</v>
       </c>
       <c r="H19" s="24" t="n">
-        <v>579</v>
+        <f aca="false">150/1</f>
+        <v>150</v>
       </c>
       <c r="I19" s="25" t="n">
         <f aca="false">IF(OR(F19="",H19=""),"",F19*H19)</f>
-        <v>579</v>
+        <v>150</v>
       </c>
       <c r="J19" s="23" t="s">
-        <v>44</v>
+        <v>31</v>
       </c>
       <c r="K19" s="26" t="s">
         <v>32</v>
@@ -2633,24 +2670,24 @@
       <c r="O19" s="30" t="s">
         <v>35</v>
       </c>
-      <c r="P19" s="31"/>
+      <c r="P19" s="31" t="s">
+        <v>69</v>
+      </c>
     </row>
     <row r="20" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="32" t="n">
         <v>10</v>
       </c>
       <c r="B20" s="33" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="C20" s="34" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="D20" s="35" t="s">
-        <v>70</v>
-      </c>
-      <c r="E20" s="21" t="s">
-        <v>71</v>
-      </c>
+        <v>72</v>
+      </c>
+      <c r="E20" s="21"/>
       <c r="F20" s="22" t="n">
         <v>1</v>
       </c>
@@ -2658,17 +2695,17 @@
         <v>30</v>
       </c>
       <c r="H20" s="24" t="n">
-        <v>100</v>
+        <v>85</v>
       </c>
       <c r="I20" s="37" t="n">
         <f aca="false">IF(OR(F20="",H20=""),"",F20*H20)</f>
-        <v>100</v>
+        <v>85</v>
       </c>
       <c r="J20" s="36" t="s">
-        <v>44</v>
+        <v>58</v>
       </c>
       <c r="K20" s="38" t="s">
-        <v>72</v>
+        <v>32</v>
       </c>
       <c r="L20" s="39" t="s">
         <v>33</v>
@@ -2676,14 +2713,12 @@
       <c r="M20" s="40" t="s">
         <v>34</v>
       </c>
-      <c r="N20" s="29" t="s">
-        <v>73</v>
-      </c>
+      <c r="N20" s="29"/>
       <c r="O20" s="30" t="s">
         <v>35</v>
       </c>
       <c r="P20" s="41" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2691,15 +2726,17 @@
         <v>11</v>
       </c>
       <c r="B21" s="18" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="C21" s="19" t="s">
+        <v>74</v>
+      </c>
+      <c r="D21" s="20" t="s">
         <v>75</v>
       </c>
-      <c r="D21" s="20" t="s">
+      <c r="E21" s="21" t="s">
         <v>76</v>
       </c>
-      <c r="E21" s="21"/>
       <c r="F21" s="22" t="n">
         <v>1</v>
       </c>
@@ -2707,17 +2744,17 @@
         <v>30</v>
       </c>
       <c r="H21" s="24" t="n">
-        <v>700</v>
+        <v>100</v>
       </c>
       <c r="I21" s="25" t="n">
         <f aca="false">IF(OR(F21="",H21=""),"",F21*H21)</f>
-        <v>700</v>
+        <v>100</v>
       </c>
       <c r="J21" s="23" t="s">
-        <v>44</v>
+        <v>31</v>
       </c>
       <c r="K21" s="26" t="s">
-        <v>72</v>
+        <v>77</v>
       </c>
       <c r="L21" s="27" t="s">
         <v>33</v>
@@ -2725,12 +2762,14 @@
       <c r="M21" s="28" t="s">
         <v>34</v>
       </c>
-      <c r="N21" s="29"/>
+      <c r="N21" s="29" t="s">
+        <v>78</v>
+      </c>
       <c r="O21" s="30" t="s">
         <v>35</v>
       </c>
       <c r="P21" s="31" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2738,13 +2777,13 @@
         <v>12</v>
       </c>
       <c r="B22" s="33" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="C22" s="34" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="D22" s="35" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="E22" s="21"/>
       <c r="F22" s="22" t="n">
@@ -2753,16 +2792,18 @@
       <c r="G22" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="H22" s="24"/>
-      <c r="I22" s="37" t="str">
+      <c r="H22" s="24" t="n">
+        <v>700</v>
+      </c>
+      <c r="I22" s="37" t="n">
         <f aca="false">IF(OR(F22="",H22=""),"",F22*H22)</f>
-        <v/>
+        <v>700</v>
       </c>
       <c r="J22" s="36" t="s">
-        <v>44</v>
+        <v>31</v>
       </c>
       <c r="K22" s="38" t="s">
-        <v>45</v>
+        <v>77</v>
       </c>
       <c r="L22" s="39" t="s">
         <v>33</v>
@@ -2775,7 +2816,7 @@
         <v>35</v>
       </c>
       <c r="P22" s="41" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2783,16 +2824,18 @@
         <v>13</v>
       </c>
       <c r="B23" s="18" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="C23" s="19" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="D23" s="20" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="E23" s="21"/>
-      <c r="F23" s="22"/>
+      <c r="F23" s="22" t="n">
+        <v>1</v>
+      </c>
       <c r="G23" s="23" t="s">
         <v>30</v>
       </c>
@@ -2802,13 +2845,13 @@
         <v/>
       </c>
       <c r="J23" s="23" t="s">
-        <v>44</v>
+        <v>31</v>
       </c>
       <c r="K23" s="26" t="s">
-        <v>64</v>
+        <v>45</v>
       </c>
       <c r="L23" s="27" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="M23" s="28" t="s">
         <v>34</v>
@@ -2818,7 +2861,7 @@
         <v>35</v>
       </c>
       <c r="P23" s="31" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2826,36 +2869,32 @@
         <v>14</v>
       </c>
       <c r="B24" s="33" t="s">
-        <v>84</v>
+        <v>70</v>
       </c>
       <c r="C24" s="34" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="D24" s="35" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="E24" s="21"/>
-      <c r="F24" s="22" t="n">
-        <v>4</v>
-      </c>
+      <c r="F24" s="22"/>
       <c r="G24" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="H24" s="24" t="n">
-        <v>37</v>
-      </c>
-      <c r="I24" s="37" t="n">
+      <c r="H24" s="24"/>
+      <c r="I24" s="37" t="str">
         <f aca="false">IF(OR(F24="",H24=""),"",F24*H24)</f>
-        <v>148</v>
+        <v/>
       </c>
       <c r="J24" s="36" t="s">
-        <v>44</v>
+        <v>31</v>
       </c>
       <c r="K24" s="38" t="s">
-        <v>72</v>
+        <v>65</v>
       </c>
       <c r="L24" s="39" t="s">
-        <v>33</v>
+        <v>41</v>
       </c>
       <c r="M24" s="40" t="s">
         <v>34</v>
@@ -2865,7 +2904,7 @@
         <v>35</v>
       </c>
       <c r="P24" s="41" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2873,13 +2912,13 @@
         <v>15</v>
       </c>
       <c r="B25" s="18" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="C25" s="19" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="D25" s="20" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="E25" s="21"/>
       <c r="F25" s="22" t="n">
@@ -2888,16 +2927,18 @@
       <c r="G25" s="23" t="s">
         <v>30</v>
       </c>
-      <c r="H25" s="24"/>
-      <c r="I25" s="25" t="str">
+      <c r="H25" s="24" t="n">
+        <v>37</v>
+      </c>
+      <c r="I25" s="25" t="n">
         <f aca="false">IF(OR(F25="",H25=""),"",F25*H25)</f>
-        <v/>
+        <v>148</v>
       </c>
       <c r="J25" s="23" t="s">
-        <v>44</v>
+        <v>31</v>
       </c>
       <c r="K25" s="26" t="s">
-        <v>45</v>
+        <v>77</v>
       </c>
       <c r="L25" s="27" t="s">
         <v>33</v>
@@ -2910,7 +2951,7 @@
         <v>35</v>
       </c>
       <c r="P25" s="31" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2918,33 +2959,31 @@
         <v>16</v>
       </c>
       <c r="B26" s="33" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="C26" s="34" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="D26" s="35" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="E26" s="21"/>
       <c r="F26" s="22" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G26" s="36" t="s">
-        <v>93</v>
-      </c>
-      <c r="H26" s="24" t="n">
-        <v>300</v>
-      </c>
-      <c r="I26" s="37" t="n">
+        <v>30</v>
+      </c>
+      <c r="H26" s="24"/>
+      <c r="I26" s="37" t="str">
         <f aca="false">IF(OR(F26="",H26=""),"",F26*H26)</f>
-        <v>300</v>
+        <v/>
       </c>
       <c r="J26" s="36" t="s">
-        <v>44</v>
+        <v>31</v>
       </c>
       <c r="K26" s="38" t="s">
-        <v>32</v>
+        <v>45</v>
       </c>
       <c r="L26" s="39" t="s">
         <v>33</v>
@@ -2956,37 +2995,39 @@
       <c r="O26" s="30" t="s">
         <v>35</v>
       </c>
-      <c r="P26" s="41"/>
+      <c r="P26" s="41" t="s">
+        <v>95</v>
+      </c>
     </row>
     <row r="27" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="17" t="n">
         <v>17</v>
       </c>
       <c r="B27" s="18" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="C27" s="19" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D27" s="20" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="E27" s="21"/>
       <c r="F27" s="22" t="n">
         <v>1</v>
       </c>
       <c r="G27" s="23" t="s">
-        <v>54</v>
+        <v>98</v>
       </c>
       <c r="H27" s="24" t="n">
-        <v>70</v>
+        <v>300</v>
       </c>
       <c r="I27" s="25" t="n">
         <f aca="false">IF(OR(F27="",H27=""),"",F27*H27)</f>
-        <v>70</v>
+        <v>300</v>
       </c>
       <c r="J27" s="23" t="s">
-        <v>44</v>
+        <v>31</v>
       </c>
       <c r="K27" s="26" t="s">
         <v>32</v>
@@ -3001,22 +3042,20 @@
       <c r="O27" s="30" t="s">
         <v>35</v>
       </c>
-      <c r="P27" s="31" t="s">
-        <v>96</v>
-      </c>
+      <c r="P27" s="31"/>
     </row>
     <row r="28" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="32" t="n">
         <v>18</v>
       </c>
       <c r="B28" s="33" t="s">
-        <v>97</v>
+        <v>89</v>
       </c>
       <c r="C28" s="34" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="D28" s="35" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="E28" s="21"/>
       <c r="F28" s="22" t="n">
@@ -3025,16 +3064,18 @@
       <c r="G28" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="H28" s="24"/>
-      <c r="I28" s="37" t="str">
+      <c r="H28" s="24" t="n">
+        <v>70</v>
+      </c>
+      <c r="I28" s="37" t="n">
         <f aca="false">IF(OR(F28="",H28=""),"",F28*H28)</f>
-        <v/>
+        <v>700</v>
       </c>
       <c r="J28" s="36" t="s">
-        <v>44</v>
+        <v>31</v>
       </c>
       <c r="K28" s="38" t="s">
-        <v>45</v>
+        <v>32</v>
       </c>
       <c r="L28" s="39" t="s">
         <v>33</v>
@@ -3047,7 +3088,7 @@
         <v>35</v>
       </c>
       <c r="P28" s="41" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3055,18 +3096,20 @@
         <v>19</v>
       </c>
       <c r="B29" s="18" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="C29" s="19" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="D29" s="20" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="E29" s="21"/>
-      <c r="F29" s="22"/>
+      <c r="F29" s="22" t="n">
+        <v>10</v>
+      </c>
       <c r="G29" s="23" t="s">
-        <v>103</v>
+        <v>30</v>
       </c>
       <c r="H29" s="24"/>
       <c r="I29" s="25" t="str">
@@ -3074,7 +3117,7 @@
         <v/>
       </c>
       <c r="J29" s="23" t="s">
-        <v>44</v>
+        <v>31</v>
       </c>
       <c r="K29" s="26" t="s">
         <v>45</v>
@@ -3090,7 +3133,7 @@
         <v>35</v>
       </c>
       <c r="P29" s="31" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3098,33 +3141,29 @@
         <v>20</v>
       </c>
       <c r="B30" s="33" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="C30" s="34" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D30" s="35" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="E30" s="21"/>
-      <c r="F30" s="22" t="n">
-        <v>1</v>
-      </c>
+      <c r="F30" s="22"/>
       <c r="G30" s="36" t="s">
-        <v>30</v>
-      </c>
-      <c r="H30" s="24" t="n">
-        <v>70</v>
-      </c>
-      <c r="I30" s="37" t="n">
+        <v>108</v>
+      </c>
+      <c r="H30" s="24"/>
+      <c r="I30" s="37" t="str">
         <f aca="false">IF(OR(F30="",H30=""),"",F30*H30)</f>
-        <v>70</v>
+        <v/>
       </c>
       <c r="J30" s="36" t="s">
-        <v>44</v>
+        <v>31</v>
       </c>
       <c r="K30" s="38" t="s">
-        <v>32</v>
+        <v>45</v>
       </c>
       <c r="L30" s="39" t="s">
         <v>33</v>
@@ -3136,20 +3175,22 @@
       <c r="O30" s="30" t="s">
         <v>35</v>
       </c>
-      <c r="P30" s="41"/>
+      <c r="P30" s="41" t="s">
+        <v>109</v>
+      </c>
     </row>
     <row r="31" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="17" t="n">
         <v>21</v>
       </c>
       <c r="B31" s="18" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="C31" s="19" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="D31" s="20" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="E31" s="21"/>
       <c r="F31" s="22" t="n">
@@ -3159,14 +3200,14 @@
         <v>30</v>
       </c>
       <c r="H31" s="24" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="I31" s="25" t="n">
         <f aca="false">IF(OR(F31="",H31=""),"",F31*H31)</f>
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="J31" s="23" t="s">
-        <v>44</v>
+        <v>31</v>
       </c>
       <c r="K31" s="26" t="s">
         <v>32</v>
@@ -3187,21 +3228,41 @@
       <c r="A32" s="32" t="n">
         <v>22</v>
       </c>
-      <c r="B32" s="33"/>
-      <c r="C32" s="34"/>
-      <c r="D32" s="35"/>
+      <c r="B32" s="33" t="s">
+        <v>102</v>
+      </c>
+      <c r="C32" s="34" t="s">
+        <v>112</v>
+      </c>
+      <c r="D32" s="35" t="s">
+        <v>113</v>
+      </c>
       <c r="E32" s="21"/>
-      <c r="F32" s="22"/>
-      <c r="G32" s="36"/>
-      <c r="H32" s="24"/>
-      <c r="I32" s="37" t="str">
+      <c r="F32" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="G32" s="36" t="s">
+        <v>30</v>
+      </c>
+      <c r="H32" s="24" t="n">
+        <v>80</v>
+      </c>
+      <c r="I32" s="37" t="n">
         <f aca="false">IF(OR(F32="",H32=""),"",F32*H32)</f>
-        <v/>
-      </c>
-      <c r="J32" s="36"/>
-      <c r="K32" s="38"/>
-      <c r="L32" s="39"/>
-      <c r="M32" s="40"/>
+        <v>80</v>
+      </c>
+      <c r="J32" s="36" t="s">
+        <v>31</v>
+      </c>
+      <c r="K32" s="38" t="s">
+        <v>32</v>
+      </c>
+      <c r="L32" s="39" t="s">
+        <v>33</v>
+      </c>
+      <c r="M32" s="40" t="s">
+        <v>34</v>
+      </c>
       <c r="N32" s="29"/>
       <c r="O32" s="30" t="s">
         <v>35</v>
@@ -3212,21 +3273,42 @@
       <c r="A33" s="17" t="n">
         <v>23</v>
       </c>
-      <c r="B33" s="18"/>
-      <c r="C33" s="19"/>
-      <c r="D33" s="20"/>
+      <c r="B33" s="18" t="s">
+        <v>102</v>
+      </c>
+      <c r="C33" s="19" t="s">
+        <v>114</v>
+      </c>
+      <c r="D33" s="20" t="s">
+        <v>115</v>
+      </c>
       <c r="E33" s="21"/>
-      <c r="F33" s="22"/>
-      <c r="G33" s="23"/>
-      <c r="H33" s="24"/>
-      <c r="I33" s="25" t="str">
+      <c r="F33" s="22" t="n">
+        <v>100</v>
+      </c>
+      <c r="G33" s="23" t="s">
+        <v>30</v>
+      </c>
+      <c r="H33" s="24" t="n">
+        <f aca="false">370/100</f>
+        <v>3.7</v>
+      </c>
+      <c r="I33" s="25" t="n">
         <f aca="false">IF(OR(F33="",H33=""),"",F33*H33)</f>
-        <v/>
-      </c>
-      <c r="J33" s="23"/>
-      <c r="K33" s="26"/>
-      <c r="L33" s="27"/>
-      <c r="M33" s="28"/>
+        <v>370</v>
+      </c>
+      <c r="J33" s="23" t="s">
+        <v>31</v>
+      </c>
+      <c r="K33" s="26" t="s">
+        <v>32</v>
+      </c>
+      <c r="L33" s="27" t="s">
+        <v>33</v>
+      </c>
+      <c r="M33" s="28" t="s">
+        <v>34</v>
+      </c>
       <c r="N33" s="29"/>
       <c r="O33" s="30" t="s">
         <v>35</v>
@@ -3308,56 +3390,106 @@
       </c>
       <c r="P36" s="41"/>
     </row>
-    <row r="37" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A37" s="1"/>
-      <c r="B37" s="1"/>
-      <c r="C37" s="42" t="s">
-        <v>109</v>
-      </c>
-      <c r="D37" s="1"/>
-      <c r="E37" s="1"/>
-      <c r="F37" s="1"/>
-      <c r="G37" s="1"/>
-      <c r="H37" s="1"/>
-      <c r="I37" s="43" t="n">
-        <f aca="false">SUMIFS($I$11:$I$36,$L$11:$L$36,"Sì")</f>
-        <v>3402.65</v>
-      </c>
-      <c r="J37" s="1"/>
-      <c r="K37" s="1"/>
-      <c r="L37" s="1"/>
-      <c r="M37" s="1"/>
-      <c r="N37" s="1"/>
-      <c r="O37" s="1"/>
-      <c r="P37" s="1"/>
-    </row>
-    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B39" s="44" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B40" s="45" t="s">
-        <v>111</v>
-      </c>
+    <row r="37" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A37" s="17" t="n">
+        <v>27</v>
+      </c>
+      <c r="B37" s="18"/>
+      <c r="C37" s="19"/>
+      <c r="D37" s="20"/>
+      <c r="E37" s="21"/>
+      <c r="F37" s="22"/>
+      <c r="G37" s="23"/>
+      <c r="H37" s="24"/>
+      <c r="I37" s="25" t="str">
+        <f aca="false">IF(OR(F37="",H37=""),"",F37*H37)</f>
+        <v/>
+      </c>
+      <c r="J37" s="23"/>
+      <c r="K37" s="26"/>
+      <c r="L37" s="27"/>
+      <c r="M37" s="28"/>
+      <c r="N37" s="29"/>
+      <c r="O37" s="30" t="s">
+        <v>35</v>
+      </c>
+      <c r="P37" s="31"/>
+    </row>
+    <row r="38" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A38" s="32" t="n">
+        <v>28</v>
+      </c>
+      <c r="B38" s="33"/>
+      <c r="C38" s="34"/>
+      <c r="D38" s="35"/>
+      <c r="E38" s="21"/>
+      <c r="F38" s="22"/>
+      <c r="G38" s="36"/>
+      <c r="H38" s="24"/>
+      <c r="I38" s="37" t="str">
+        <f aca="false">IF(OR(F38="",H38=""),"",F38*H38)</f>
+        <v/>
+      </c>
+      <c r="J38" s="36"/>
+      <c r="K38" s="38"/>
+      <c r="L38" s="39"/>
+      <c r="M38" s="40"/>
+      <c r="N38" s="29"/>
+      <c r="O38" s="30" t="s">
+        <v>35</v>
+      </c>
+      <c r="P38" s="41"/>
+    </row>
+    <row r="39" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A39" s="1"/>
+      <c r="B39" s="1"/>
+      <c r="C39" s="42" t="s">
+        <v>116</v>
+      </c>
+      <c r="D39" s="1"/>
+      <c r="E39" s="1"/>
+      <c r="F39" s="1"/>
+      <c r="G39" s="1"/>
+      <c r="H39" s="1"/>
+      <c r="I39" s="43" t="n">
+        <f aca="false">SUMIFS($I$11:$I$38,$L$11:$L$38,"Sì")</f>
+        <v>4537</v>
+      </c>
+      <c r="J39" s="1"/>
+      <c r="K39" s="1"/>
+      <c r="L39" s="1"/>
+      <c r="M39" s="1"/>
+      <c r="N39" s="1"/>
+      <c r="O39" s="1"/>
+      <c r="P39" s="1"/>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B41" s="45" t="s">
-        <v>112</v>
+      <c r="B41" s="44" t="s">
+        <v>117</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B42" s="45" t="s">
-        <v>113</v>
+        <v>118</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B43" s="45" t="s">
-        <v>114</v>
+        <v>119</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B44" s="45" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B45" s="45" t="s">
+        <v>121</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A10:P36"/>
+  <autoFilter ref="A10:P38"/>
   <mergeCells count="10">
     <mergeCell ref="B5:C5"/>
     <mergeCell ref="E5:G5"/>
@@ -3370,7 +3502,7 @@
     <mergeCell ref="J6:L6"/>
     <mergeCell ref="M6:N6"/>
   </mergeCells>
-  <conditionalFormatting sqref="K11:K36">
+  <conditionalFormatting sqref="K11:K38">
     <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="19">
       <formula>$K11="Preventivo"</formula>
     </cfRule>
@@ -3387,7 +3519,7 @@
       <formula>$K11="Da definire"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="M11:M36">
+  <conditionalFormatting sqref="M11:M38">
     <cfRule type="expression" priority="7" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="24">
       <formula>$M11="Ordinato"</formula>
     </cfRule>
@@ -3398,28 +3530,28 @@
       <formula>$M11="Pagato"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I11:I36">
+  <conditionalFormatting sqref="I11:I38">
     <cfRule type="expression" priority="10" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="27">
       <formula>$L11="No"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="3">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="K11:K36" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="K11:K38" type="list">
       <formula1>"Preventivo,Stima,Opzionale,Alternativa,Da definire"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="L11:L36" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="L11:L38" type="list">
       <formula1>"Sì,No"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="M11:M36" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="M11:M38" type="list">
       <formula1>"Da ordinare,Ordinato,Consegnato,Pagato"</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
   <hyperlinks>
     <hyperlink ref="N15" r:id="rId2" display="golflags.eu"/>
-    <hyperlink ref="N20" r:id="rId3" display="amazon.it"/>
+    <hyperlink ref="N21" r:id="rId3" display="amazon.it"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="true" verticalCentered="false"/>
   <pageMargins left="0.4" right="0.4" top="1" bottom="1" header="0.511811023622047" footer="0.5"/>
@@ -3452,7 +3584,7 @@
     <row r="1" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1"/>
       <c r="B1" s="46" t="s">
-        <v>115</v>
+        <v>122</v>
       </c>
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
@@ -3463,7 +3595,7 @@
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1"/>
       <c r="B2" s="47" t="s">
-        <v>116</v>
+        <v>123</v>
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
@@ -3477,7 +3609,7 @@
         <v>12</v>
       </c>
       <c r="C4" s="48" t="s">
-        <v>117</v>
+        <v>124</v>
       </c>
       <c r="D4" s="48" t="s">
         <v>3</v>
@@ -3489,147 +3621,147 @@
         <v>19</v>
       </c>
       <c r="G4" s="48" t="s">
-        <v>118</v>
+        <v>125</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="50" t="s">
-        <v>119</v>
+        <v>126</v>
       </c>
       <c r="B5" s="51" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="C5" s="52" t="n">
-        <f aca="false">COUNTIFS('Piano di spesa'!$B$11:$B$36,"A · Stampa e comunicazione")</f>
+        <f aca="false">COUNTIFS('Piano di spesa'!$B$11:$B$38,"A · Stampa e comunicazione")</f>
         <v>4</v>
       </c>
       <c r="D5" s="53" t="n">
-        <f aca="false">SUMIFS('Piano di spesa'!$I$11:$I$36,'Piano di spesa'!$B$11:$B$36,"A · Stampa e comunicazione",'Piano di spesa'!$L$11:$L$36,"Sì")</f>
-        <v>311.65</v>
+        <f aca="false">SUMIFS('Piano di spesa'!$I$11:$I$38,'Piano di spesa'!$B$11:$B$38,"A · Stampa e comunicazione",'Piano di spesa'!$L$11:$L$38,"Sì")</f>
+        <v>420</v>
       </c>
       <c r="E5" s="54" t="n">
-        <f aca="false">SUMIFS('Piano di spesa'!$I$11:$I$36,'Piano di spesa'!$B$11:$B$36,"A · Stampa e comunicazione",'Piano di spesa'!$K$11:$K$36,"Opzionale",'Piano di spesa'!$L$11:$L$36,"No")</f>
+        <f aca="false">SUMIFS('Piano di spesa'!$I$11:$I$38,'Piano di spesa'!$B$11:$B$38,"A · Stampa e comunicazione",'Piano di spesa'!$K$11:$K$38,"Opzionale",'Piano di spesa'!$L$11:$L$38,"No")</f>
         <v>0</v>
       </c>
       <c r="F5" s="54" t="n">
         <f aca="false">D5+E5</f>
-        <v>311.65</v>
+        <v>420</v>
       </c>
       <c r="G5" s="55" t="n">
         <f aca="false">IF($D$10=0,0,D5/$D$10)</f>
-        <v>0.091590378087667</v>
+        <v>0.0925721842627287</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="50" t="s">
-        <v>121</v>
+        <v>128</v>
       </c>
       <c r="B6" s="51" t="s">
-        <v>122</v>
+        <v>129</v>
       </c>
       <c r="C6" s="52" t="n">
-        <f aca="false">COUNTIFS('Piano di spesa'!$B$11:$B$36,"B · Allestimento del campo")</f>
-        <v>4</v>
+        <f aca="false">COUNTIFS('Piano di spesa'!$B$11:$B$38,"B · Allestimento del campo")</f>
+        <v>5</v>
       </c>
       <c r="D6" s="53" t="n">
-        <f aca="false">SUMIFS('Piano di spesa'!$I$11:$I$36,'Piano di spesa'!$B$11:$B$36,"B · Allestimento del campo",'Piano di spesa'!$L$11:$L$36,"Sì")</f>
-        <v>1044</v>
+        <f aca="false">SUMIFS('Piano di spesa'!$I$11:$I$38,'Piano di spesa'!$B$11:$B$38,"B · Allestimento del campo",'Piano di spesa'!$L$11:$L$38,"Sì")</f>
+        <v>1564</v>
       </c>
       <c r="E6" s="54" t="n">
-        <f aca="false">SUMIFS('Piano di spesa'!$I$11:$I$36,'Piano di spesa'!$B$11:$B$36,"B · Allestimento del campo",'Piano di spesa'!$K$11:$K$36,"Opzionale",'Piano di spesa'!$L$11:$L$36,"No")</f>
+        <f aca="false">SUMIFS('Piano di spesa'!$I$11:$I$38,'Piano di spesa'!$B$11:$B$38,"B · Allestimento del campo",'Piano di spesa'!$K$11:$K$38,"Opzionale",'Piano di spesa'!$L$11:$L$38,"No")</f>
         <v>2000</v>
       </c>
       <c r="F6" s="54" t="n">
         <f aca="false">D6+E6</f>
-        <v>3044</v>
+        <v>3564</v>
       </c>
       <c r="G6" s="55" t="n">
         <f aca="false">IF($D$10=0,0,D6/$D$10)</f>
-        <v>0.306819684657546</v>
+        <v>0.344721181397399</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="50" t="s">
-        <v>123</v>
+        <v>130</v>
       </c>
       <c r="B7" s="51" t="s">
-        <v>124</v>
+        <v>131</v>
       </c>
       <c r="C7" s="52" t="n">
-        <f aca="false">COUNTIFS('Piano di spesa'!$B$11:$B$36,"C · Immagine, media e presentazione")</f>
+        <f aca="false">COUNTIFS('Piano di spesa'!$B$11:$B$38,"C · Immagine, media e presentazione")</f>
         <v>5</v>
       </c>
       <c r="D7" s="53" t="n">
-        <f aca="false">SUMIFS('Piano di spesa'!$I$11:$I$36,'Piano di spesa'!$B$11:$B$36,"C · Immagine, media e presentazione",'Piano di spesa'!$L$11:$L$36,"Sì")</f>
-        <v>1379</v>
+        <f aca="false">SUMIFS('Piano di spesa'!$I$11:$I$38,'Piano di spesa'!$B$11:$B$38,"C · Immagine, media e presentazione",'Piano di spesa'!$L$11:$L$38,"Sì")</f>
+        <v>885</v>
       </c>
       <c r="E7" s="54" t="n">
-        <f aca="false">SUMIFS('Piano di spesa'!$I$11:$I$36,'Piano di spesa'!$B$11:$B$36,"C · Immagine, media e presentazione",'Piano di spesa'!$K$11:$K$36,"Opzionale",'Piano di spesa'!$L$11:$L$36,"No")</f>
+        <f aca="false">SUMIFS('Piano di spesa'!$I$11:$I$38,'Piano di spesa'!$B$11:$B$38,"C · Immagine, media e presentazione",'Piano di spesa'!$K$11:$K$38,"Opzionale",'Piano di spesa'!$L$11:$L$38,"No")</f>
         <v>0</v>
       </c>
       <c r="F7" s="54" t="n">
         <f aca="false">D7+E7</f>
-        <v>1379</v>
+        <v>885</v>
       </c>
       <c r="G7" s="55" t="n">
         <f aca="false">IF($D$10=0,0,D7/$D$10)</f>
-        <v>0.405272361247851</v>
+        <v>0.195062816839321</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="50" t="s">
-        <v>125</v>
+        <v>132</v>
       </c>
       <c r="B8" s="51" t="s">
-        <v>126</v>
+        <v>133</v>
       </c>
       <c r="C8" s="52" t="n">
-        <f aca="false">COUNTIFS('Piano di spesa'!$B$11:$B$36,"D · Accoglienza e punto ristoro")</f>
+        <f aca="false">COUNTIFS('Piano di spesa'!$B$11:$B$38,"D · Accoglienza e punto ristoro")</f>
         <v>4</v>
       </c>
       <c r="D8" s="53" t="n">
-        <f aca="false">SUMIFS('Piano di spesa'!$I$11:$I$36,'Piano di spesa'!$B$11:$B$36,"D · Accoglienza e punto ristoro",'Piano di spesa'!$L$11:$L$36,"Sì")</f>
-        <v>518</v>
+        <f aca="false">SUMIFS('Piano di spesa'!$I$11:$I$38,'Piano di spesa'!$B$11:$B$38,"D · Accoglienza e punto ristoro",'Piano di spesa'!$L$11:$L$38,"Sì")</f>
+        <v>1148</v>
       </c>
       <c r="E8" s="54" t="n">
-        <f aca="false">SUMIFS('Piano di spesa'!$I$11:$I$36,'Piano di spesa'!$B$11:$B$36,"D · Accoglienza e punto ristoro",'Piano di spesa'!$K$11:$K$36,"Opzionale",'Piano di spesa'!$L$11:$L$36,"No")</f>
+        <f aca="false">SUMIFS('Piano di spesa'!$I$11:$I$38,'Piano di spesa'!$B$11:$B$38,"D · Accoglienza e punto ristoro",'Piano di spesa'!$K$11:$K$38,"Opzionale",'Piano di spesa'!$L$11:$L$38,"No")</f>
         <v>0</v>
       </c>
       <c r="F8" s="54" t="n">
         <f aca="false">D8+E8</f>
-        <v>518</v>
+        <v>1148</v>
       </c>
       <c r="G8" s="55" t="n">
         <f aca="false">IF($D$10=0,0,D8/$D$10)</f>
-        <v>0.152234287981426</v>
+        <v>0.253030636984792</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="50" t="s">
-        <v>127</v>
+        <v>134</v>
       </c>
       <c r="B9" s="51" t="s">
-        <v>128</v>
+        <v>135</v>
       </c>
       <c r="C9" s="52" t="n">
-        <f aca="false">COUNTIFS('Piano di spesa'!$B$11:$B$36,"E · Organizzazione e staff")</f>
-        <v>4</v>
+        <f aca="false">COUNTIFS('Piano di spesa'!$B$11:$B$38,"E · Organizzazione e staff")</f>
+        <v>5</v>
       </c>
       <c r="D9" s="53" t="n">
-        <f aca="false">SUMIFS('Piano di spesa'!$I$11:$I$36,'Piano di spesa'!$B$11:$B$36,"E · Organizzazione e staff",'Piano di spesa'!$L$11:$L$36,"Sì")</f>
-        <v>150</v>
+        <f aca="false">SUMIFS('Piano di spesa'!$I$11:$I$38,'Piano di spesa'!$B$11:$B$38,"E · Organizzazione e staff",'Piano di spesa'!$L$11:$L$38,"Sì")</f>
+        <v>520</v>
       </c>
       <c r="E9" s="54" t="n">
-        <f aca="false">SUMIFS('Piano di spesa'!$I$11:$I$36,'Piano di spesa'!$B$11:$B$36,"E · Organizzazione e staff",'Piano di spesa'!$K$11:$K$36,"Opzionale",'Piano di spesa'!$L$11:$L$36,"No")</f>
+        <f aca="false">SUMIFS('Piano di spesa'!$I$11:$I$38,'Piano di spesa'!$B$11:$B$38,"E · Organizzazione e staff",'Piano di spesa'!$K$11:$K$38,"Opzionale",'Piano di spesa'!$L$11:$L$38,"No")</f>
         <v>0</v>
       </c>
       <c r="F9" s="54" t="n">
         <f aca="false">D9+E9</f>
-        <v>150</v>
+        <v>520</v>
       </c>
       <c r="G9" s="55" t="n">
         <f aca="false">IF($D$10=0,0,D9/$D$10)</f>
-        <v>0.0440832880255095</v>
+        <v>0.114613180515759</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3639,11 +3771,11 @@
       </c>
       <c r="C10" s="57" t="n">
         <f aca="false">SUM(C5:C9)</f>
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="D10" s="58" t="n">
         <f aca="false">SUM(D5:D9)</f>
-        <v>3402.65</v>
+        <v>4537</v>
       </c>
       <c r="E10" s="59" t="n">
         <f aca="false">SUM(E5:E9)</f>
@@ -3651,7 +3783,7 @@
       </c>
       <c r="F10" s="59" t="n">
         <f aca="false">SUM(F5:F9)</f>
-        <v>5402.65</v>
+        <v>6537</v>
       </c>
       <c r="G10" s="60" t="n">
         <f aca="false">IF($D$10=0,0,SUM(G5:G9))</f>

</xml_diff>

<commit_message>
Piano di spesa Tappa Zero: cubi e drone opzionali, sedie € 70 in tutto
Cubi in polionda e drone passano fra le voci eventuali, fuori dal totale base;
le 10 sedie per gazebo costano € 70 complessive. Le etichette degli opzionali
si ricavano dalle voci. Totale base € 3.057, opzionali € 2.850.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014EyPNYo6uPPTyzbFJvdbw6
</commit_message>
<xml_diff>
--- a/piano-spesa-tappa-zero-2026/dist/piano-spesa-tappa-zero-2026.xlsx
+++ b/piano-spesa-tappa-zero-2026/dist/piano-spesa-tappa-zero-2026.xlsx
@@ -66,6 +66,18 @@
         </r>
       </text>
     </comment>
+    <comment ref="H28" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Dal preventivo: € 70,00 complessivi per 10 pz,</t>
+        </r>
+      </text>
+    </comment>
     <comment ref="H33" authorId="0">
       <text>
         <r>
@@ -304,7 +316,7 @@
     <t xml:space="preserve">Cubi in polionda 5 mm, 30 × 30 cm.</t>
   </si>
   <si>
-    <t xml:space="preserve">Verificare quanti cubi comprende la fornitura.</t>
+    <t xml:space="preserve">Voce eventuale, fuori dal totale base. Verificare quanti cubi comprende la fornitura.</t>
   </si>
   <si>
     <t xml:space="preserve">C · Immagine, media e presentazione</t>
@@ -343,7 +355,7 @@
     <t xml:space="preserve">DJI Mini 4 Pro o Mini 5 Pro per riprese aeree e diretta streaming della tappa.</t>
   </si>
   <si>
-    <t xml:space="preserve">€ 400–700 secondo modello e kit: messo il massimo per prudenza.</t>
+    <t xml:space="preserve">Voce eventuale, fuori dal totale base. € 400–700 secondo modello: messo il massimo.</t>
   </si>
   <si>
     <t xml:space="preserve">Tovaglia tavolo AIFG</t>
@@ -400,7 +412,7 @@
     <t xml:space="preserve">Sedie per i gazebo dell'accoglienza e della segreteria.</t>
   </si>
   <si>
-    <t xml:space="preserve">€ 70 a sedia.</t>
+    <t xml:space="preserve">€ 70 in tutto per le 10 sedie.</t>
   </si>
   <si>
     <t xml:space="preserve">E · Organizzazione e staff</t>
@@ -454,7 +466,7 @@
     <t xml:space="preserve">• Brochure (n. 1) e pieghevole A3 (n. 2) sono alternativi: nel totale base c'è la brochure. Per passare all'A3 invertire «Nel totale» sulle due righe.</t>
   </si>
   <si>
-    <t xml:space="preserve">• Mini vele (n. 8) è voce eventuale, fuori dal totale base. Telo proiettore (€ 80–100) e drone (€ 400–700): messo il massimo per prudenza.</t>
+    <t xml:space="preserve">• Mini vele, cubi e drone sono voci eventuali, fuori dal totale base. Telo proiettore (€ 80–100) e drone (€ 400–700): messo il massimo per prudenza.</t>
   </si>
   <si>
     <t xml:space="preserve">• Tavoli ristoro: quantità 4 ipotizzata, da confermare. IVA «Esclusa» o «Inclusa» solo dove il preventivo lo dice: altrimenti da verificare.</t>
@@ -1674,13 +1686,13 @@
                   <c:v>420</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>1564</c:v>
+                  <c:v>1414</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>885</c:v>
+                  <c:v>185</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>1148</c:v>
+                  <c:v>518</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>520</c:v>
@@ -1691,11 +1703,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="67172425"/>
-        <c:axId val="23899440"/>
+        <c:axId val="49202488"/>
+        <c:axId val="69618189"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="67172425"/>
+        <c:axId val="49202488"/>
         <c:scaling>
           <c:orientation val="maxMin"/>
         </c:scaling>
@@ -1727,7 +1739,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="23899440"/>
+        <c:crossAx val="69618189"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1735,7 +1747,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="23899440"/>
+        <c:axId val="69618189"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1767,7 +1779,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="67172425"/>
+        <c:crossAx val="49202488"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2163,16 +2175,16 @@
     <row r="6" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B6" s="7" t="n">
         <f aca="false">SUMIFS($I$11:$I$38,$L$11:$L$38,"Sì")</f>
-        <v>4537</v>
+        <v>3057</v>
       </c>
       <c r="C6" s="7"/>
       <c r="D6" s="8" t="n">
         <f aca="false">SUMIFS($I$11:$I$38,$K$11:$K$38,"Opzionale",$L$11:$L$38,"No")</f>
-        <v>2000</v>
+        <v>2850</v>
       </c>
       <c r="E6" s="9" t="n">
         <f aca="false">B6+D6</f>
-        <v>6537</v>
+        <v>5907</v>
       </c>
       <c r="F6" s="9"/>
       <c r="G6" s="9"/>
@@ -2658,10 +2670,10 @@
         <v>31</v>
       </c>
       <c r="K19" s="26" t="s">
-        <v>32</v>
+        <v>65</v>
       </c>
       <c r="L19" s="27" t="s">
-        <v>33</v>
+        <v>41</v>
       </c>
       <c r="M19" s="28" t="s">
         <v>34</v>
@@ -2803,10 +2815,10 @@
         <v>31</v>
       </c>
       <c r="K22" s="38" t="s">
-        <v>77</v>
+        <v>65</v>
       </c>
       <c r="L22" s="39" t="s">
-        <v>33</v>
+        <v>41</v>
       </c>
       <c r="M22" s="40" t="s">
         <v>34</v>
@@ -3065,11 +3077,12 @@
         <v>30</v>
       </c>
       <c r="H28" s="24" t="n">
-        <v>70</v>
+        <f aca="false">70/10</f>
+        <v>7</v>
       </c>
       <c r="I28" s="37" t="n">
         <f aca="false">IF(OR(F28="",H28=""),"",F28*H28)</f>
-        <v>700</v>
+        <v>70</v>
       </c>
       <c r="J28" s="36" t="s">
         <v>31</v>
@@ -3453,7 +3466,7 @@
       <c r="H39" s="1"/>
       <c r="I39" s="43" t="n">
         <f aca="false">SUMIFS($I$11:$I$38,$L$11:$L$38,"Sì")</f>
-        <v>4537</v>
+        <v>3057</v>
       </c>
       <c r="J39" s="1"/>
       <c r="K39" s="1"/>
@@ -3649,7 +3662,7 @@
       </c>
       <c r="G5" s="55" t="n">
         <f aca="false">IF($D$10=0,0,D5/$D$10)</f>
-        <v>0.0925721842627287</v>
+        <v>0.13738959764475</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3665,11 +3678,11 @@
       </c>
       <c r="D6" s="53" t="n">
         <f aca="false">SUMIFS('Piano di spesa'!$I$11:$I$38,'Piano di spesa'!$B$11:$B$38,"B · Allestimento del campo",'Piano di spesa'!$L$11:$L$38,"Sì")</f>
-        <v>1564</v>
+        <v>1414</v>
       </c>
       <c r="E6" s="54" t="n">
         <f aca="false">SUMIFS('Piano di spesa'!$I$11:$I$38,'Piano di spesa'!$B$11:$B$38,"B · Allestimento del campo",'Piano di spesa'!$K$11:$K$38,"Opzionale",'Piano di spesa'!$L$11:$L$38,"No")</f>
-        <v>2000</v>
+        <v>2150</v>
       </c>
       <c r="F6" s="54" t="n">
         <f aca="false">D6+E6</f>
@@ -3677,7 +3690,7 @@
       </c>
       <c r="G6" s="55" t="n">
         <f aca="false">IF($D$10=0,0,D6/$D$10)</f>
-        <v>0.344721181397399</v>
+        <v>0.462544978737324</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3693,11 +3706,11 @@
       </c>
       <c r="D7" s="53" t="n">
         <f aca="false">SUMIFS('Piano di spesa'!$I$11:$I$38,'Piano di spesa'!$B$11:$B$38,"C · Immagine, media e presentazione",'Piano di spesa'!$L$11:$L$38,"Sì")</f>
-        <v>885</v>
+        <v>185</v>
       </c>
       <c r="E7" s="54" t="n">
         <f aca="false">SUMIFS('Piano di spesa'!$I$11:$I$38,'Piano di spesa'!$B$11:$B$38,"C · Immagine, media e presentazione",'Piano di spesa'!$K$11:$K$38,"Opzionale",'Piano di spesa'!$L$11:$L$38,"No")</f>
-        <v>0</v>
+        <v>700</v>
       </c>
       <c r="F7" s="54" t="n">
         <f aca="false">D7+E7</f>
@@ -3705,7 +3718,7 @@
       </c>
       <c r="G7" s="55" t="n">
         <f aca="false">IF($D$10=0,0,D7/$D$10)</f>
-        <v>0.195062816839321</v>
+        <v>0.060516846581616</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3721,7 +3734,7 @@
       </c>
       <c r="D8" s="53" t="n">
         <f aca="false">SUMIFS('Piano di spesa'!$I$11:$I$38,'Piano di spesa'!$B$11:$B$38,"D · Accoglienza e punto ristoro",'Piano di spesa'!$L$11:$L$38,"Sì")</f>
-        <v>1148</v>
+        <v>518</v>
       </c>
       <c r="E8" s="54" t="n">
         <f aca="false">SUMIFS('Piano di spesa'!$I$11:$I$38,'Piano di spesa'!$B$11:$B$38,"D · Accoglienza e punto ristoro",'Piano di spesa'!$K$11:$K$38,"Opzionale",'Piano di spesa'!$L$11:$L$38,"No")</f>
@@ -3729,11 +3742,11 @@
       </c>
       <c r="F8" s="54" t="n">
         <f aca="false">D8+E8</f>
-        <v>1148</v>
+        <v>518</v>
       </c>
       <c r="G8" s="55" t="n">
         <f aca="false">IF($D$10=0,0,D8/$D$10)</f>
-        <v>0.253030636984792</v>
+        <v>0.169447170428525</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3761,7 +3774,7 @@
       </c>
       <c r="G9" s="55" t="n">
         <f aca="false">IF($D$10=0,0,D9/$D$10)</f>
-        <v>0.114613180515759</v>
+        <v>0.170101406607785</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3775,15 +3788,15 @@
       </c>
       <c r="D10" s="58" t="n">
         <f aca="false">SUM(D5:D9)</f>
-        <v>4537</v>
+        <v>3057</v>
       </c>
       <c r="E10" s="59" t="n">
         <f aca="false">SUM(E5:E9)</f>
-        <v>2000</v>
+        <v>2850</v>
       </c>
       <c r="F10" s="59" t="n">
         <f aca="false">SUM(F5:F9)</f>
-        <v>6537</v>
+        <v>5907</v>
       </c>
       <c r="G10" s="60" t="n">
         <f aca="false">IF($D$10=0,0,SUM(G5:G9))</f>

</xml_diff>